<commit_message>
Sheets API: accept bare array or {rows}, 400 on bad bodies, validate tool ids, server-side formula evaluation on GET (Python + no-eval JS engine for Workers), optimistic locking (base_updated_at/If-Match -> 409), login rate limiting, per-user currency/offer-type settings; stage-aware ad diagnosis; one value-gap rule; cash exposure + winner recency + sell-existing-product-first; separate market vs creator ladders; CSV rounding, multi-sheet XLSX import, tab names, weekly-review formula rows, Start-here path; CLI sheet commands; tests
</commit_message>
<xml_diff>
--- a/templates/xlsx/ad-diagnosis.xlsx
+++ b/templates/xlsx/ad-diagnosis.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paid Ads Diagnosis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -566,7 +566,7 @@
         <v/>
       </c>
       <c r="J2" s="6">
-        <f>IF(A2="","",IF(D2=0,"Check target/activation",IF(C2="Seed","P2 keep (seeding)",IF(H2&gt;=G2,"P2 hero - scale",IF(H2&gt;=G2*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A2="","",IF(D2=0,"Check target/activation",IF(C2="Seed","P2 keep (seeding)",IF(H2&gt;=G2,"P2 hero - scale",IF(AND(B2="0→1 validate",F2&lt;50),"Learning - hold until ~50 conversions",IF(H2&gt;=G2*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -583,7 +583,7 @@
         <v/>
       </c>
       <c r="J3" s="6">
-        <f>IF(A3="","",IF(D3=0,"Check target/activation",IF(C3="Seed","P2 keep (seeding)",IF(H3&gt;=G3,"P2 hero - scale",IF(H3&gt;=G3*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A3="","",IF(D3=0,"Check target/activation",IF(C3="Seed","P2 keep (seeding)",IF(H3&gt;=G3,"P2 hero - scale",IF(AND(B3="0→1 validate",F3&lt;50),"Learning - hold until ~50 conversions",IF(H3&gt;=G3*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -600,7 +600,7 @@
         <v/>
       </c>
       <c r="J4" s="6">
-        <f>IF(A4="","",IF(D4=0,"Check target/activation",IF(C4="Seed","P2 keep (seeding)",IF(H4&gt;=G4,"P2 hero - scale",IF(H4&gt;=G4*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A4="","",IF(D4=0,"Check target/activation",IF(C4="Seed","P2 keep (seeding)",IF(H4&gt;=G4,"P2 hero - scale",IF(AND(B4="0→1 validate",F4&lt;50),"Learning - hold until ~50 conversions",IF(H4&gt;=G4*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -617,7 +617,7 @@
         <v/>
       </c>
       <c r="J5" s="6">
-        <f>IF(A5="","",IF(D5=0,"Check target/activation",IF(C5="Seed","P2 keep (seeding)",IF(H5&gt;=G5,"P2 hero - scale",IF(H5&gt;=G5*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A5="","",IF(D5=0,"Check target/activation",IF(C5="Seed","P2 keep (seeding)",IF(H5&gt;=G5,"P2 hero - scale",IF(AND(B5="0→1 validate",F5&lt;50),"Learning - hold until ~50 conversions",IF(H5&gt;=G5*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -634,7 +634,7 @@
         <v/>
       </c>
       <c r="J6" s="6">
-        <f>IF(A6="","",IF(D6=0,"Check target/activation",IF(C6="Seed","P2 keep (seeding)",IF(H6&gt;=G6,"P2 hero - scale",IF(H6&gt;=G6*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A6="","",IF(D6=0,"Check target/activation",IF(C6="Seed","P2 keep (seeding)",IF(H6&gt;=G6,"P2 hero - scale",IF(AND(B6="0→1 validate",F6&lt;50),"Learning - hold until ~50 conversions",IF(H6&gt;=G6*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -651,7 +651,7 @@
         <v/>
       </c>
       <c r="J7" s="6">
-        <f>IF(A7="","",IF(D7=0,"Check target/activation",IF(C7="Seed","P2 keep (seeding)",IF(H7&gt;=G7,"P2 hero - scale",IF(H7&gt;=G7*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A7="","",IF(D7=0,"Check target/activation",IF(C7="Seed","P2 keep (seeding)",IF(H7&gt;=G7,"P2 hero - scale",IF(AND(B7="0→1 validate",F7&lt;50),"Learning - hold until ~50 conversions",IF(H7&gt;=G7*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -668,7 +668,7 @@
         <v/>
       </c>
       <c r="J8" s="6">
-        <f>IF(A8="","",IF(D8=0,"Check target/activation",IF(C8="Seed","P2 keep (seeding)",IF(H8&gt;=G8,"P2 hero - scale",IF(H8&gt;=G8*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A8="","",IF(D8=0,"Check target/activation",IF(C8="Seed","P2 keep (seeding)",IF(H8&gt;=G8,"P2 hero - scale",IF(AND(B8="0→1 validate",F8&lt;50),"Learning - hold until ~50 conversions",IF(H8&gt;=G8*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -685,7 +685,7 @@
         <v/>
       </c>
       <c r="J9" s="6">
-        <f>IF(A9="","",IF(D9=0,"Check target/activation",IF(C9="Seed","P2 keep (seeding)",IF(H9&gt;=G9,"P2 hero - scale",IF(H9&gt;=G9*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A9="","",IF(D9=0,"Check target/activation",IF(C9="Seed","P2 keep (seeding)",IF(H9&gt;=G9,"P2 hero - scale",IF(AND(B9="0→1 validate",F9&lt;50),"Learning - hold until ~50 conversions",IF(H9&gt;=G9*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         <v/>
       </c>
       <c r="J10" s="6">
-        <f>IF(A10="","",IF(D10=0,"Check target/activation",IF(C10="Seed","P2 keep (seeding)",IF(H10&gt;=G10,"P2 hero - scale",IF(H10&gt;=G10*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A10="","",IF(D10=0,"Check target/activation",IF(C10="Seed","P2 keep (seeding)",IF(H10&gt;=G10,"P2 hero - scale",IF(AND(B10="0→1 validate",F10&lt;50),"Learning - hold until ~50 conversions",IF(H10&gt;=G10*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -719,7 +719,7 @@
         <v/>
       </c>
       <c r="J11" s="6">
-        <f>IF(A11="","",IF(D11=0,"Check target/activation",IF(C11="Seed","P2 keep (seeding)",IF(H11&gt;=G11,"P2 hero - scale",IF(H11&gt;=G11*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A11="","",IF(D11=0,"Check target/activation",IF(C11="Seed","P2 keep (seeding)",IF(H11&gt;=G11,"P2 hero - scale",IF(AND(B11="0→1 validate",F11&lt;50),"Learning - hold until ~50 conversions",IF(H11&gt;=G11*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -736,7 +736,7 @@
         <v/>
       </c>
       <c r="J12" s="6">
-        <f>IF(A12="","",IF(D12=0,"Check target/activation",IF(C12="Seed","P2 keep (seeding)",IF(H12&gt;=G12,"P2 hero - scale",IF(H12&gt;=G12*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A12="","",IF(D12=0,"Check target/activation",IF(C12="Seed","P2 keep (seeding)",IF(H12&gt;=G12,"P2 hero - scale",IF(AND(B12="0→1 validate",F12&lt;50),"Learning - hold until ~50 conversions",IF(H12&gt;=G12*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -753,7 +753,7 @@
         <v/>
       </c>
       <c r="J13" s="6">
-        <f>IF(A13="","",IF(D13=0,"Check target/activation",IF(C13="Seed","P2 keep (seeding)",IF(H13&gt;=G13,"P2 hero - scale",IF(H13&gt;=G13*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A13="","",IF(D13=0,"Check target/activation",IF(C13="Seed","P2 keep (seeding)",IF(H13&gt;=G13,"P2 hero - scale",IF(AND(B13="0→1 validate",F13&lt;50),"Learning - hold until ~50 conversions",IF(H13&gt;=G13*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -770,7 +770,7 @@
         <v/>
       </c>
       <c r="J14" s="6">
-        <f>IF(A14="","",IF(D14=0,"Check target/activation",IF(C14="Seed","P2 keep (seeding)",IF(H14&gt;=G14,"P2 hero - scale",IF(H14&gt;=G14*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A14="","",IF(D14=0,"Check target/activation",IF(C14="Seed","P2 keep (seeding)",IF(H14&gt;=G14,"P2 hero - scale",IF(AND(B14="0→1 validate",F14&lt;50),"Learning - hold until ~50 conversions",IF(H14&gt;=G14*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -787,7 +787,7 @@
         <v/>
       </c>
       <c r="J15" s="6">
-        <f>IF(A15="","",IF(D15=0,"Check target/activation",IF(C15="Seed","P2 keep (seeding)",IF(H15&gt;=G15,"P2 hero - scale",IF(H15&gt;=G15*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A15="","",IF(D15=0,"Check target/activation",IF(C15="Seed","P2 keep (seeding)",IF(H15&gt;=G15,"P2 hero - scale",IF(AND(B15="0→1 validate",F15&lt;50),"Learning - hold until ~50 conversions",IF(H15&gt;=G15*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -804,7 +804,7 @@
         <v/>
       </c>
       <c r="J16" s="6">
-        <f>IF(A16="","",IF(D16=0,"Check target/activation",IF(C16="Seed","P2 keep (seeding)",IF(H16&gt;=G16,"P2 hero - scale",IF(H16&gt;=G16*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A16="","",IF(D16=0,"Check target/activation",IF(C16="Seed","P2 keep (seeding)",IF(H16&gt;=G16,"P2 hero - scale",IF(AND(B16="0→1 validate",F16&lt;50),"Learning - hold until ~50 conversions",IF(H16&gt;=G16*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -821,7 +821,7 @@
         <v/>
       </c>
       <c r="J17" s="6">
-        <f>IF(A17="","",IF(D17=0,"Check target/activation",IF(C17="Seed","P2 keep (seeding)",IF(H17&gt;=G17,"P2 hero - scale",IF(H17&gt;=G17*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A17="","",IF(D17=0,"Check target/activation",IF(C17="Seed","P2 keep (seeding)",IF(H17&gt;=G17,"P2 hero - scale",IF(AND(B17="0→1 validate",F17&lt;50),"Learning - hold until ~50 conversions",IF(H17&gt;=G17*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -838,7 +838,7 @@
         <v/>
       </c>
       <c r="J18" s="6">
-        <f>IF(A18="","",IF(D18=0,"Check target/activation",IF(C18="Seed","P2 keep (seeding)",IF(H18&gt;=G18,"P2 hero - scale",IF(H18&gt;=G18*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A18="","",IF(D18=0,"Check target/activation",IF(C18="Seed","P2 keep (seeding)",IF(H18&gt;=G18,"P2 hero - scale",IF(AND(B18="0→1 validate",F18&lt;50),"Learning - hold until ~50 conversions",IF(H18&gt;=G18*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -855,7 +855,7 @@
         <v/>
       </c>
       <c r="J19" s="6">
-        <f>IF(A19="","",IF(D19=0,"Check target/activation",IF(C19="Seed","P2 keep (seeding)",IF(H19&gt;=G19,"P2 hero - scale",IF(H19&gt;=G19*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A19="","",IF(D19=0,"Check target/activation",IF(C19="Seed","P2 keep (seeding)",IF(H19&gt;=G19,"P2 hero - scale",IF(AND(B19="0→1 validate",F19&lt;50),"Learning - hold until ~50 conversions",IF(H19&gt;=G19*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -872,7 +872,7 @@
         <v/>
       </c>
       <c r="J20" s="6">
-        <f>IF(A20="","",IF(D20=0,"Check target/activation",IF(C20="Seed","P2 keep (seeding)",IF(H20&gt;=G20,"P2 hero - scale",IF(H20&gt;=G20*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A20="","",IF(D20=0,"Check target/activation",IF(C20="Seed","P2 keep (seeding)",IF(H20&gt;=G20,"P2 hero - scale",IF(AND(B20="0→1 validate",F20&lt;50),"Learning - hold until ~50 conversions",IF(H20&gt;=G20*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -889,7 +889,7 @@
         <v/>
       </c>
       <c r="J21" s="6">
-        <f>IF(A21="","",IF(D21=0,"Check target/activation",IF(C21="Seed","P2 keep (seeding)",IF(H21&gt;=G21,"P2 hero - scale",IF(H21&gt;=G21*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A21="","",IF(D21=0,"Check target/activation",IF(C21="Seed","P2 keep (seeding)",IF(H21&gt;=G21,"P2 hero - scale",IF(AND(B21="0→1 validate",F21&lt;50),"Learning - hold until ~50 conversions",IF(H21&gt;=G21*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -906,7 +906,7 @@
         <v/>
       </c>
       <c r="J22" s="6">
-        <f>IF(A22="","",IF(D22=0,"Check target/activation",IF(C22="Seed","P2 keep (seeding)",IF(H22&gt;=G22,"P2 hero - scale",IF(H22&gt;=G22*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A22="","",IF(D22=0,"Check target/activation",IF(C22="Seed","P2 keep (seeding)",IF(H22&gt;=G22,"P2 hero - scale",IF(AND(B22="0→1 validate",F22&lt;50),"Learning - hold until ~50 conversions",IF(H22&gt;=G22*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -923,7 +923,7 @@
         <v/>
       </c>
       <c r="J23" s="6">
-        <f>IF(A23="","",IF(D23=0,"Check target/activation",IF(C23="Seed","P2 keep (seeding)",IF(H23&gt;=G23,"P2 hero - scale",IF(H23&gt;=G23*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A23="","",IF(D23=0,"Check target/activation",IF(C23="Seed","P2 keep (seeding)",IF(H23&gt;=G23,"P2 hero - scale",IF(AND(B23="0→1 validate",F23&lt;50),"Learning - hold until ~50 conversions",IF(H23&gt;=G23*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -940,7 +940,7 @@
         <v/>
       </c>
       <c r="J24" s="6">
-        <f>IF(A24="","",IF(D24=0,"Check target/activation",IF(C24="Seed","P2 keep (seeding)",IF(H24&gt;=G24,"P2 hero - scale",IF(H24&gt;=G24*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A24="","",IF(D24=0,"Check target/activation",IF(C24="Seed","P2 keep (seeding)",IF(H24&gt;=G24,"P2 hero - scale",IF(AND(B24="0→1 validate",F24&lt;50),"Learning - hold until ~50 conversions",IF(H24&gt;=G24*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -957,7 +957,7 @@
         <v/>
       </c>
       <c r="J25" s="6">
-        <f>IF(A25="","",IF(D25=0,"Check target/activation",IF(C25="Seed","P2 keep (seeding)",IF(H25&gt;=G25,"P2 hero - scale",IF(H25&gt;=G25*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A25="","",IF(D25=0,"Check target/activation",IF(C25="Seed","P2 keep (seeding)",IF(H25&gt;=G25,"P2 hero - scale",IF(AND(B25="0→1 validate",F25&lt;50),"Learning - hold until ~50 conversions",IF(H25&gt;=G25*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v/>
       </c>
       <c r="J26" s="6">
-        <f>IF(A26="","",IF(D26=0,"Check target/activation",IF(C26="Seed","P2 keep (seeding)",IF(H26&gt;=G26,"P2 hero - scale",IF(H26&gt;=G26*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A26="","",IF(D26=0,"Check target/activation",IF(C26="Seed","P2 keep (seeding)",IF(H26&gt;=G26,"P2 hero - scale",IF(AND(B26="0→1 validate",F26&lt;50),"Learning - hold until ~50 conversions",IF(H26&gt;=G26*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -991,7 +991,7 @@
         <v/>
       </c>
       <c r="J27" s="6">
-        <f>IF(A27="","",IF(D27=0,"Check target/activation",IF(C27="Seed","P2 keep (seeding)",IF(H27&gt;=G27,"P2 hero - scale",IF(H27&gt;=G27*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A27="","",IF(D27=0,"Check target/activation",IF(C27="Seed","P2 keep (seeding)",IF(H27&gt;=G27,"P2 hero - scale",IF(AND(B27="0→1 validate",F27&lt;50),"Learning - hold until ~50 conversions",IF(H27&gt;=G27*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
         <v/>
       </c>
       <c r="J28" s="6">
-        <f>IF(A28="","",IF(D28=0,"Check target/activation",IF(C28="Seed","P2 keep (seeding)",IF(H28&gt;=G28,"P2 hero - scale",IF(H28&gt;=G28*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A28="","",IF(D28=0,"Check target/activation",IF(C28="Seed","P2 keep (seeding)",IF(H28&gt;=G28,"P2 hero - scale",IF(AND(B28="0→1 validate",F28&lt;50),"Learning - hold until ~50 conversions",IF(H28&gt;=G28*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
         <v/>
       </c>
       <c r="J29" s="6">
-        <f>IF(A29="","",IF(D29=0,"Check target/activation",IF(C29="Seed","P2 keep (seeding)",IF(H29&gt;=G29,"P2 hero - scale",IF(H29&gt;=G29*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A29="","",IF(D29=0,"Check target/activation",IF(C29="Seed","P2 keep (seeding)",IF(H29&gt;=G29,"P2 hero - scale",IF(AND(B29="0→1 validate",F29&lt;50),"Learning - hold until ~50 conversions",IF(H29&gt;=G29*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
         <v/>
       </c>
       <c r="J30" s="6">
-        <f>IF(A30="","",IF(D30=0,"Check target/activation",IF(C30="Seed","P2 keep (seeding)",IF(H30&gt;=G30,"P2 hero - scale",IF(H30&gt;=G30*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A30="","",IF(D30=0,"Check target/activation",IF(C30="Seed","P2 keep (seeding)",IF(H30&gt;=G30,"P2 hero - scale",IF(AND(B30="0→1 validate",F30&lt;50),"Learning - hold until ~50 conversions",IF(H30&gt;=G30*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
         <v/>
       </c>
       <c r="J31" s="6">
-        <f>IF(A31="","",IF(D31=0,"Check target/activation",IF(C31="Seed","P2 keep (seeding)",IF(H31&gt;=G31,"P2 hero - scale",IF(H31&gt;=G31*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A31="","",IF(D31=0,"Check target/activation",IF(C31="Seed","P2 keep (seeding)",IF(H31&gt;=G31,"P2 hero - scale",IF(AND(B31="0→1 validate",F31&lt;50),"Learning - hold until ~50 conversions",IF(H31&gt;=G31*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
         <v/>
       </c>
       <c r="J32" s="6">
-        <f>IF(A32="","",IF(D32=0,"Check target/activation",IF(C32="Seed","P2 keep (seeding)",IF(H32&gt;=G32,"P2 hero - scale",IF(H32&gt;=G32*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A32="","",IF(D32=0,"Check target/activation",IF(C32="Seed","P2 keep (seeding)",IF(H32&gt;=G32,"P2 hero - scale",IF(AND(B32="0→1 validate",F32&lt;50),"Learning - hold until ~50 conversions",IF(H32&gt;=G32*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
         <v/>
       </c>
       <c r="J33" s="6">
-        <f>IF(A33="","",IF(D33=0,"Check target/activation",IF(C33="Seed","P2 keep (seeding)",IF(H33&gt;=G33,"P2 hero - scale",IF(H33&gt;=G33*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A33="","",IF(D33=0,"Check target/activation",IF(C33="Seed","P2 keep (seeding)",IF(H33&gt;=G33,"P2 hero - scale",IF(AND(B33="0→1 validate",F33&lt;50),"Learning - hold until ~50 conversions",IF(H33&gt;=G33*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
         <v/>
       </c>
       <c r="J34" s="6">
-        <f>IF(A34="","",IF(D34=0,"Check target/activation",IF(C34="Seed","P2 keep (seeding)",IF(H34&gt;=G34,"P2 hero - scale",IF(H34&gt;=G34*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A34="","",IF(D34=0,"Check target/activation",IF(C34="Seed","P2 keep (seeding)",IF(H34&gt;=G34,"P2 hero - scale",IF(AND(B34="0→1 validate",F34&lt;50),"Learning - hold until ~50 conversions",IF(H34&gt;=G34*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
       <c r="J35" s="6">
-        <f>IF(A35="","",IF(D35=0,"Check target/activation",IF(C35="Seed","P2 keep (seeding)",IF(H35&gt;=G35,"P2 hero - scale",IF(H35&gt;=G35*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A35="","",IF(D35=0,"Check target/activation",IF(C35="Seed","P2 keep (seeding)",IF(H35&gt;=G35,"P2 hero - scale",IF(AND(B35="0→1 validate",F35&lt;50),"Learning - hold until ~50 conversions",IF(H35&gt;=G35*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
         <v/>
       </c>
       <c r="J36" s="6">
-        <f>IF(A36="","",IF(D36=0,"Check target/activation",IF(C36="Seed","P2 keep (seeding)",IF(H36&gt;=G36,"P2 hero - scale",IF(H36&gt;=G36*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A36="","",IF(D36=0,"Check target/activation",IF(C36="Seed","P2 keep (seeding)",IF(H36&gt;=G36,"P2 hero - scale",IF(AND(B36="0→1 validate",F36&lt;50),"Learning - hold until ~50 conversions",IF(H36&gt;=G36*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
         <v/>
       </c>
       <c r="J37" s="6">
-        <f>IF(A37="","",IF(D37=0,"Check target/activation",IF(C37="Seed","P2 keep (seeding)",IF(H37&gt;=G37,"P2 hero - scale",IF(H37&gt;=G37*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A37="","",IF(D37=0,"Check target/activation",IF(C37="Seed","P2 keep (seeding)",IF(H37&gt;=G37,"P2 hero - scale",IF(AND(B37="0→1 validate",F37&lt;50),"Learning - hold until ~50 conversions",IF(H37&gt;=G37*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
         <v/>
       </c>
       <c r="J38" s="6">
-        <f>IF(A38="","",IF(D38=0,"Check target/activation",IF(C38="Seed","P2 keep (seeding)",IF(H38&gt;=G38,"P2 hero - scale",IF(H38&gt;=G38*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A38="","",IF(D38=0,"Check target/activation",IF(C38="Seed","P2 keep (seeding)",IF(H38&gt;=G38,"P2 hero - scale",IF(AND(B38="0→1 validate",F38&lt;50),"Learning - hold until ~50 conversions",IF(H38&gt;=G38*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
         <v/>
       </c>
       <c r="J39" s="6">
-        <f>IF(A39="","",IF(D39=0,"Check target/activation",IF(C39="Seed","P2 keep (seeding)",IF(H39&gt;=G39,"P2 hero - scale",IF(H39&gt;=G39*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A39="","",IF(D39=0,"Check target/activation",IF(C39="Seed","P2 keep (seeding)",IF(H39&gt;=G39,"P2 hero - scale",IF(AND(B39="0→1 validate",F39&lt;50),"Learning - hold until ~50 conversions",IF(H39&gt;=G39*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         <v/>
       </c>
       <c r="J40" s="6">
-        <f>IF(A40="","",IF(D40=0,"Check target/activation",IF(C40="Seed","P2 keep (seeding)",IF(H40&gt;=G40,"P2 hero - scale",IF(H40&gt;=G40*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A40="","",IF(D40=0,"Check target/activation",IF(C40="Seed","P2 keep (seeding)",IF(H40&gt;=G40,"P2 hero - scale",IF(AND(B40="0→1 validate",F40&lt;50),"Learning - hold until ~50 conversions",IF(H40&gt;=G40*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
         <v/>
       </c>
       <c r="J41" s="6">
-        <f>IF(A41="","",IF(D41=0,"Check target/activation",IF(C41="Seed","P2 keep (seeding)",IF(H41&gt;=G41,"P2 hero - scale",IF(H41&gt;=G41*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A41="","",IF(D41=0,"Check target/activation",IF(C41="Seed","P2 keep (seeding)",IF(H41&gt;=G41,"P2 hero - scale",IF(AND(B41="0→1 validate",F41&lt;50),"Learning - hold until ~50 conversions",IF(H41&gt;=G41*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
         <v/>
       </c>
       <c r="J42" s="6">
-        <f>IF(A42="","",IF(D42=0,"Check target/activation",IF(C42="Seed","P2 keep (seeding)",IF(H42&gt;=G42,"P2 hero - scale",IF(H42&gt;=G42*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A42="","",IF(D42=0,"Check target/activation",IF(C42="Seed","P2 keep (seeding)",IF(H42&gt;=G42,"P2 hero - scale",IF(AND(B42="0→1 validate",F42&lt;50),"Learning - hold until ~50 conversions",IF(H42&gt;=G42*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
         <v/>
       </c>
       <c r="J43" s="6">
-        <f>IF(A43="","",IF(D43=0,"Check target/activation",IF(C43="Seed","P2 keep (seeding)",IF(H43&gt;=G43,"P2 hero - scale",IF(H43&gt;=G43*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A43="","",IF(D43=0,"Check target/activation",IF(C43="Seed","P2 keep (seeding)",IF(H43&gt;=G43,"P2 hero - scale",IF(AND(B43="0→1 validate",F43&lt;50),"Learning - hold until ~50 conversions",IF(H43&gt;=G43*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="J44" s="6">
-        <f>IF(A44="","",IF(D44=0,"Check target/activation",IF(C44="Seed","P2 keep (seeding)",IF(H44&gt;=G44,"P2 hero - scale",IF(H44&gt;=G44*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A44="","",IF(D44=0,"Check target/activation",IF(C44="Seed","P2 keep (seeding)",IF(H44&gt;=G44,"P2 hero - scale",IF(AND(B44="0→1 validate",F44&lt;50),"Learning - hold until ~50 conversions",IF(H44&gt;=G44*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
         <v/>
       </c>
       <c r="J45" s="6">
-        <f>IF(A45="","",IF(D45=0,"Check target/activation",IF(C45="Seed","P2 keep (seeding)",IF(H45&gt;=G45,"P2 hero - scale",IF(H45&gt;=G45*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A45="","",IF(D45=0,"Check target/activation",IF(C45="Seed","P2 keep (seeding)",IF(H45&gt;=G45,"P2 hero - scale",IF(AND(B45="0→1 validate",F45&lt;50),"Learning - hold until ~50 conversions",IF(H45&gt;=G45*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
         <v/>
       </c>
       <c r="J46" s="6">
-        <f>IF(A46="","",IF(D46=0,"Check target/activation",IF(C46="Seed","P2 keep (seeding)",IF(H46&gt;=G46,"P2 hero - scale",IF(H46&gt;=G46*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A46="","",IF(D46=0,"Check target/activation",IF(C46="Seed","P2 keep (seeding)",IF(H46&gt;=G46,"P2 hero - scale",IF(AND(B46="0→1 validate",F46&lt;50),"Learning - hold until ~50 conversions",IF(H46&gt;=G46*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
         <v/>
       </c>
       <c r="J47" s="6">
-        <f>IF(A47="","",IF(D47=0,"Check target/activation",IF(C47="Seed","P2 keep (seeding)",IF(H47&gt;=G47,"P2 hero - scale",IF(H47&gt;=G47*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A47="","",IF(D47=0,"Check target/activation",IF(C47="Seed","P2 keep (seeding)",IF(H47&gt;=G47,"P2 hero - scale",IF(AND(B47="0→1 validate",F47&lt;50),"Learning - hold until ~50 conversions",IF(H47&gt;=G47*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
         <v/>
       </c>
       <c r="J48" s="6">
-        <f>IF(A48="","",IF(D48=0,"Check target/activation",IF(C48="Seed","P2 keep (seeding)",IF(H48&gt;=G48,"P2 hero - scale",IF(H48&gt;=G48*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A48="","",IF(D48=0,"Check target/activation",IF(C48="Seed","P2 keep (seeding)",IF(H48&gt;=G48,"P2 hero - scale",IF(AND(B48="0→1 validate",F48&lt;50),"Learning - hold until ~50 conversions",IF(H48&gt;=G48*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1365,7 +1365,7 @@
         <v/>
       </c>
       <c r="J49" s="6">
-        <f>IF(A49="","",IF(D49=0,"Check target/activation",IF(C49="Seed","P2 keep (seeding)",IF(H49&gt;=G49,"P2 hero - scale",IF(H49&gt;=G49*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A49="","",IF(D49=0,"Check target/activation",IF(C49="Seed","P2 keep (seeding)",IF(H49&gt;=G49,"P2 hero - scale",IF(AND(B49="0→1 validate",F49&lt;50),"Learning - hold until ~50 conversions",IF(H49&gt;=G49*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
         <v/>
       </c>
       <c r="J50" s="6">
-        <f>IF(A50="","",IF(D50=0,"Check target/activation",IF(C50="Seed","P2 keep (seeding)",IF(H50&gt;=G50,"P2 hero - scale",IF(H50&gt;=G50*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A50="","",IF(D50=0,"Check target/activation",IF(C50="Seed","P2 keep (seeding)",IF(H50&gt;=G50,"P2 hero - scale",IF(AND(B50="0→1 validate",F50&lt;50),"Learning - hold until ~50 conversions",IF(H50&gt;=G50*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
         <v/>
       </c>
       <c r="J51" s="6">
-        <f>IF(A51="","",IF(D51=0,"Check target/activation",IF(C51="Seed","P2 keep (seeding)",IF(H51&gt;=G51,"P2 hero - scale",IF(H51&gt;=G51*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A51="","",IF(D51=0,"Check target/activation",IF(C51="Seed","P2 keep (seeding)",IF(H51&gt;=G51,"P2 hero - scale",IF(AND(B51="0→1 validate",F51&lt;50),"Learning - hold until ~50 conversions",IF(H51&gt;=G51*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
         <v/>
       </c>
       <c r="J52" s="6">
-        <f>IF(A52="","",IF(D52=0,"Check target/activation",IF(C52="Seed","P2 keep (seeding)",IF(H52&gt;=G52,"P2 hero - scale",IF(H52&gt;=G52*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A52="","",IF(D52=0,"Check target/activation",IF(C52="Seed","P2 keep (seeding)",IF(H52&gt;=G52,"P2 hero - scale",IF(AND(B52="0→1 validate",F52&lt;50),"Learning - hold until ~50 conversions",IF(H52&gt;=G52*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
         <v/>
       </c>
       <c r="J53" s="6">
-        <f>IF(A53="","",IF(D53=0,"Check target/activation",IF(C53="Seed","P2 keep (seeding)",IF(H53&gt;=G53,"P2 hero - scale",IF(H53&gt;=G53*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A53="","",IF(D53=0,"Check target/activation",IF(C53="Seed","P2 keep (seeding)",IF(H53&gt;=G53,"P2 hero - scale",IF(AND(B53="0→1 validate",F53&lt;50),"Learning - hold until ~50 conversions",IF(H53&gt;=G53*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1450,7 +1450,7 @@
         <v/>
       </c>
       <c r="J54" s="6">
-        <f>IF(A54="","",IF(D54=0,"Check target/activation",IF(C54="Seed","P2 keep (seeding)",IF(H54&gt;=G54,"P2 hero - scale",IF(H54&gt;=G54*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A54="","",IF(D54=0,"Check target/activation",IF(C54="Seed","P2 keep (seeding)",IF(H54&gt;=G54,"P2 hero - scale",IF(AND(B54="0→1 validate",F54&lt;50),"Learning - hold until ~50 conversions",IF(H54&gt;=G54*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
         <v/>
       </c>
       <c r="J55" s="6">
-        <f>IF(A55="","",IF(D55=0,"Check target/activation",IF(C55="Seed","P2 keep (seeding)",IF(H55&gt;=G55,"P2 hero - scale",IF(H55&gt;=G55*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A55="","",IF(D55=0,"Check target/activation",IF(C55="Seed","P2 keep (seeding)",IF(H55&gt;=G55,"P2 hero - scale",IF(AND(B55="0→1 validate",F55&lt;50),"Learning - hold until ~50 conversions",IF(H55&gt;=G55*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
         <v/>
       </c>
       <c r="J56" s="6">
-        <f>IF(A56="","",IF(D56=0,"Check target/activation",IF(C56="Seed","P2 keep (seeding)",IF(H56&gt;=G56,"P2 hero - scale",IF(H56&gt;=G56*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A56="","",IF(D56=0,"Check target/activation",IF(C56="Seed","P2 keep (seeding)",IF(H56&gt;=G56,"P2 hero - scale",IF(AND(B56="0→1 validate",F56&lt;50),"Learning - hold until ~50 conversions",IF(H56&gt;=G56*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
         <v/>
       </c>
       <c r="J57" s="6">
-        <f>IF(A57="","",IF(D57=0,"Check target/activation",IF(C57="Seed","P2 keep (seeding)",IF(H57&gt;=G57,"P2 hero - scale",IF(H57&gt;=G57*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A57="","",IF(D57=0,"Check target/activation",IF(C57="Seed","P2 keep (seeding)",IF(H57&gt;=G57,"P2 hero - scale",IF(AND(B57="0→1 validate",F57&lt;50),"Learning - hold until ~50 conversions",IF(H57&gt;=G57*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
         <v/>
       </c>
       <c r="J58" s="6">
-        <f>IF(A58="","",IF(D58=0,"Check target/activation",IF(C58="Seed","P2 keep (seeding)",IF(H58&gt;=G58,"P2 hero - scale",IF(H58&gt;=G58*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A58="","",IF(D58=0,"Check target/activation",IF(C58="Seed","P2 keep (seeding)",IF(H58&gt;=G58,"P2 hero - scale",IF(AND(B58="0→1 validate",F58&lt;50),"Learning - hold until ~50 conversions",IF(H58&gt;=G58*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
         <v/>
       </c>
       <c r="J59" s="6">
-        <f>IF(A59="","",IF(D59=0,"Check target/activation",IF(C59="Seed","P2 keep (seeding)",IF(H59&gt;=G59,"P2 hero - scale",IF(H59&gt;=G59*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A59="","",IF(D59=0,"Check target/activation",IF(C59="Seed","P2 keep (seeding)",IF(H59&gt;=G59,"P2 hero - scale",IF(AND(B59="0→1 validate",F59&lt;50),"Learning - hold until ~50 conversions",IF(H59&gt;=G59*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1552,7 +1552,7 @@
         <v/>
       </c>
       <c r="J60" s="6">
-        <f>IF(A60="","",IF(D60=0,"Check target/activation",IF(C60="Seed","P2 keep (seeding)",IF(H60&gt;=G60,"P2 hero - scale",IF(H60&gt;=G60*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A60="","",IF(D60=0,"Check target/activation",IF(C60="Seed","P2 keep (seeding)",IF(H60&gt;=G60,"P2 hero - scale",IF(AND(B60="0→1 validate",F60&lt;50),"Learning - hold until ~50 conversions",IF(H60&gt;=G60*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
         <v/>
       </c>
       <c r="J61" s="6">
-        <f>IF(A61="","",IF(D61=0,"Check target/activation",IF(C61="Seed","P2 keep (seeding)",IF(H61&gt;=G61,"P2 hero - scale",IF(H61&gt;=G61*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A61="","",IF(D61=0,"Check target/activation",IF(C61="Seed","P2 keep (seeding)",IF(H61&gt;=G61,"P2 hero - scale",IF(AND(B61="0→1 validate",F61&lt;50),"Learning - hold until ~50 conversions",IF(H61&gt;=G61*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
         <v/>
       </c>
       <c r="J62" s="6">
-        <f>IF(A62="","",IF(D62=0,"Check target/activation",IF(C62="Seed","P2 keep (seeding)",IF(H62&gt;=G62,"P2 hero - scale",IF(H62&gt;=G62*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A62="","",IF(D62=0,"Check target/activation",IF(C62="Seed","P2 keep (seeding)",IF(H62&gt;=G62,"P2 hero - scale",IF(AND(B62="0→1 validate",F62&lt;50),"Learning - hold until ~50 conversions",IF(H62&gt;=G62*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1603,7 +1603,7 @@
         <v/>
       </c>
       <c r="J63" s="6">
-        <f>IF(A63="","",IF(D63=0,"Check target/activation",IF(C63="Seed","P2 keep (seeding)",IF(H63&gt;=G63,"P2 hero - scale",IF(H63&gt;=G63*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A63="","",IF(D63=0,"Check target/activation",IF(C63="Seed","P2 keep (seeding)",IF(H63&gt;=G63,"P2 hero - scale",IF(AND(B63="0→1 validate",F63&lt;50),"Learning - hold until ~50 conversions",IF(H63&gt;=G63*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
         <v/>
       </c>
       <c r="J64" s="6">
-        <f>IF(A64="","",IF(D64=0,"Check target/activation",IF(C64="Seed","P2 keep (seeding)",IF(H64&gt;=G64,"P2 hero - scale",IF(H64&gt;=G64*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A64="","",IF(D64=0,"Check target/activation",IF(C64="Seed","P2 keep (seeding)",IF(H64&gt;=G64,"P2 hero - scale",IF(AND(B64="0→1 validate",F64&lt;50),"Learning - hold until ~50 conversions",IF(H64&gt;=G64*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
         <v/>
       </c>
       <c r="J65" s="6">
-        <f>IF(A65="","",IF(D65=0,"Check target/activation",IF(C65="Seed","P2 keep (seeding)",IF(H65&gt;=G65,"P2 hero - scale",IF(H65&gt;=G65*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A65="","",IF(D65=0,"Check target/activation",IF(C65="Seed","P2 keep (seeding)",IF(H65&gt;=G65,"P2 hero - scale",IF(AND(B65="0→1 validate",F65&lt;50),"Learning - hold until ~50 conversions",IF(H65&gt;=G65*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
         <v/>
       </c>
       <c r="J66" s="6">
-        <f>IF(A66="","",IF(D66=0,"Check target/activation",IF(C66="Seed","P2 keep (seeding)",IF(H66&gt;=G66,"P2 hero - scale",IF(H66&gt;=G66*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A66="","",IF(D66=0,"Check target/activation",IF(C66="Seed","P2 keep (seeding)",IF(H66&gt;=G66,"P2 hero - scale",IF(AND(B66="0→1 validate",F66&lt;50),"Learning - hold until ~50 conversions",IF(H66&gt;=G66*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
         <v/>
       </c>
       <c r="J67" s="6">
-        <f>IF(A67="","",IF(D67=0,"Check target/activation",IF(C67="Seed","P2 keep (seeding)",IF(H67&gt;=G67,"P2 hero - scale",IF(H67&gt;=G67*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A67="","",IF(D67=0,"Check target/activation",IF(C67="Seed","P2 keep (seeding)",IF(H67&gt;=G67,"P2 hero - scale",IF(AND(B67="0→1 validate",F67&lt;50),"Learning - hold until ~50 conversions",IF(H67&gt;=G67*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
         <v/>
       </c>
       <c r="J68" s="6">
-        <f>IF(A68="","",IF(D68=0,"Check target/activation",IF(C68="Seed","P2 keep (seeding)",IF(H68&gt;=G68,"P2 hero - scale",IF(H68&gt;=G68*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A68="","",IF(D68=0,"Check target/activation",IF(C68="Seed","P2 keep (seeding)",IF(H68&gt;=G68,"P2 hero - scale",IF(AND(B68="0→1 validate",F68&lt;50),"Learning - hold until ~50 conversions",IF(H68&gt;=G68*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1705,7 +1705,7 @@
         <v/>
       </c>
       <c r="J69" s="6">
-        <f>IF(A69="","",IF(D69=0,"Check target/activation",IF(C69="Seed","P2 keep (seeding)",IF(H69&gt;=G69,"P2 hero - scale",IF(H69&gt;=G69*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A69="","",IF(D69=0,"Check target/activation",IF(C69="Seed","P2 keep (seeding)",IF(H69&gt;=G69,"P2 hero - scale",IF(AND(B69="0→1 validate",F69&lt;50),"Learning - hold until ~50 conversions",IF(H69&gt;=G69*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1722,7 +1722,7 @@
         <v/>
       </c>
       <c r="J70" s="6">
-        <f>IF(A70="","",IF(D70=0,"Check target/activation",IF(C70="Seed","P2 keep (seeding)",IF(H70&gt;=G70,"P2 hero - scale",IF(H70&gt;=G70*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A70="","",IF(D70=0,"Check target/activation",IF(C70="Seed","P2 keep (seeding)",IF(H70&gt;=G70,"P2 hero - scale",IF(AND(B70="0→1 validate",F70&lt;50),"Learning - hold until ~50 conversions",IF(H70&gt;=G70*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1739,7 +1739,7 @@
         <v/>
       </c>
       <c r="J71" s="6">
-        <f>IF(A71="","",IF(D71=0,"Check target/activation",IF(C71="Seed","P2 keep (seeding)",IF(H71&gt;=G71,"P2 hero - scale",IF(H71&gt;=G71*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A71="","",IF(D71=0,"Check target/activation",IF(C71="Seed","P2 keep (seeding)",IF(H71&gt;=G71,"P2 hero - scale",IF(AND(B71="0→1 validate",F71&lt;50),"Learning - hold until ~50 conversions",IF(H71&gt;=G71*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
         <v/>
       </c>
       <c r="J72" s="6">
-        <f>IF(A72="","",IF(D72=0,"Check target/activation",IF(C72="Seed","P2 keep (seeding)",IF(H72&gt;=G72,"P2 hero - scale",IF(H72&gt;=G72*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A72="","",IF(D72=0,"Check target/activation",IF(C72="Seed","P2 keep (seeding)",IF(H72&gt;=G72,"P2 hero - scale",IF(AND(B72="0→1 validate",F72&lt;50),"Learning - hold until ~50 conversions",IF(H72&gt;=G72*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
         <v/>
       </c>
       <c r="J73" s="6">
-        <f>IF(A73="","",IF(D73=0,"Check target/activation",IF(C73="Seed","P2 keep (seeding)",IF(H73&gt;=G73,"P2 hero - scale",IF(H73&gt;=G73*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A73="","",IF(D73=0,"Check target/activation",IF(C73="Seed","P2 keep (seeding)",IF(H73&gt;=G73,"P2 hero - scale",IF(AND(B73="0→1 validate",F73&lt;50),"Learning - hold until ~50 conversions",IF(H73&gt;=G73*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
         <v/>
       </c>
       <c r="J74" s="6">
-        <f>IF(A74="","",IF(D74=0,"Check target/activation",IF(C74="Seed","P2 keep (seeding)",IF(H74&gt;=G74,"P2 hero - scale",IF(H74&gt;=G74*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A74="","",IF(D74=0,"Check target/activation",IF(C74="Seed","P2 keep (seeding)",IF(H74&gt;=G74,"P2 hero - scale",IF(AND(B74="0→1 validate",F74&lt;50),"Learning - hold until ~50 conversions",IF(H74&gt;=G74*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
         <v/>
       </c>
       <c r="J75" s="6">
-        <f>IF(A75="","",IF(D75=0,"Check target/activation",IF(C75="Seed","P2 keep (seeding)",IF(H75&gt;=G75,"P2 hero - scale",IF(H75&gt;=G75*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A75="","",IF(D75=0,"Check target/activation",IF(C75="Seed","P2 keep (seeding)",IF(H75&gt;=G75,"P2 hero - scale",IF(AND(B75="0→1 validate",F75&lt;50),"Learning - hold until ~50 conversions",IF(H75&gt;=G75*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
         <v/>
       </c>
       <c r="J76" s="6">
-        <f>IF(A76="","",IF(D76=0,"Check target/activation",IF(C76="Seed","P2 keep (seeding)",IF(H76&gt;=G76,"P2 hero - scale",IF(H76&gt;=G76*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A76="","",IF(D76=0,"Check target/activation",IF(C76="Seed","P2 keep (seeding)",IF(H76&gt;=G76,"P2 hero - scale",IF(AND(B76="0→1 validate",F76&lt;50),"Learning - hold until ~50 conversions",IF(H76&gt;=G76*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
         <v/>
       </c>
       <c r="J77" s="6">
-        <f>IF(A77="","",IF(D77=0,"Check target/activation",IF(C77="Seed","P2 keep (seeding)",IF(H77&gt;=G77,"P2 hero - scale",IF(H77&gt;=G77*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A77="","",IF(D77=0,"Check target/activation",IF(C77="Seed","P2 keep (seeding)",IF(H77&gt;=G77,"P2 hero - scale",IF(AND(B77="0→1 validate",F77&lt;50),"Learning - hold until ~50 conversions",IF(H77&gt;=G77*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
         <v/>
       </c>
       <c r="J78" s="6">
-        <f>IF(A78="","",IF(D78=0,"Check target/activation",IF(C78="Seed","P2 keep (seeding)",IF(H78&gt;=G78,"P2 hero - scale",IF(H78&gt;=G78*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A78="","",IF(D78=0,"Check target/activation",IF(C78="Seed","P2 keep (seeding)",IF(H78&gt;=G78,"P2 hero - scale",IF(AND(B78="0→1 validate",F78&lt;50),"Learning - hold until ~50 conversions",IF(H78&gt;=G78*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1875,7 +1875,7 @@
         <v/>
       </c>
       <c r="J79" s="6">
-        <f>IF(A79="","",IF(D79=0,"Check target/activation",IF(C79="Seed","P2 keep (seeding)",IF(H79&gt;=G79,"P2 hero - scale",IF(H79&gt;=G79*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A79="","",IF(D79=0,"Check target/activation",IF(C79="Seed","P2 keep (seeding)",IF(H79&gt;=G79,"P2 hero - scale",IF(AND(B79="0→1 validate",F79&lt;50),"Learning - hold until ~50 conversions",IF(H79&gt;=G79*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
         <v/>
       </c>
       <c r="J80" s="6">
-        <f>IF(A80="","",IF(D80=0,"Check target/activation",IF(C80="Seed","P2 keep (seeding)",IF(H80&gt;=G80,"P2 hero - scale",IF(H80&gt;=G80*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A80="","",IF(D80=0,"Check target/activation",IF(C80="Seed","P2 keep (seeding)",IF(H80&gt;=G80,"P2 hero - scale",IF(AND(B80="0→1 validate",F80&lt;50),"Learning - hold until ~50 conversions",IF(H80&gt;=G80*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
         <v/>
       </c>
       <c r="J81" s="6">
-        <f>IF(A81="","",IF(D81=0,"Check target/activation",IF(C81="Seed","P2 keep (seeding)",IF(H81&gt;=G81,"P2 hero - scale",IF(H81&gt;=G81*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A81="","",IF(D81=0,"Check target/activation",IF(C81="Seed","P2 keep (seeding)",IF(H81&gt;=G81,"P2 hero - scale",IF(AND(B81="0→1 validate",F81&lt;50),"Learning - hold until ~50 conversions",IF(H81&gt;=G81*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
         <v/>
       </c>
       <c r="J82" s="6">
-        <f>IF(A82="","",IF(D82=0,"Check target/activation",IF(C82="Seed","P2 keep (seeding)",IF(H82&gt;=G82,"P2 hero - scale",IF(H82&gt;=G82*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A82="","",IF(D82=0,"Check target/activation",IF(C82="Seed","P2 keep (seeding)",IF(H82&gt;=G82,"P2 hero - scale",IF(AND(B82="0→1 validate",F82&lt;50),"Learning - hold until ~50 conversions",IF(H82&gt;=G82*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
         <v/>
       </c>
       <c r="J83" s="6">
-        <f>IF(A83="","",IF(D83=0,"Check target/activation",IF(C83="Seed","P2 keep (seeding)",IF(H83&gt;=G83,"P2 hero - scale",IF(H83&gt;=G83*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A83="","",IF(D83=0,"Check target/activation",IF(C83="Seed","P2 keep (seeding)",IF(H83&gt;=G83,"P2 hero - scale",IF(AND(B83="0→1 validate",F83&lt;50),"Learning - hold until ~50 conversions",IF(H83&gt;=G83*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
         <v/>
       </c>
       <c r="J84" s="6">
-        <f>IF(A84="","",IF(D84=0,"Check target/activation",IF(C84="Seed","P2 keep (seeding)",IF(H84&gt;=G84,"P2 hero - scale",IF(H84&gt;=G84*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A84="","",IF(D84=0,"Check target/activation",IF(C84="Seed","P2 keep (seeding)",IF(H84&gt;=G84,"P2 hero - scale",IF(AND(B84="0→1 validate",F84&lt;50),"Learning - hold until ~50 conversions",IF(H84&gt;=G84*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
         <v/>
       </c>
       <c r="J85" s="6">
-        <f>IF(A85="","",IF(D85=0,"Check target/activation",IF(C85="Seed","P2 keep (seeding)",IF(H85&gt;=G85,"P2 hero - scale",IF(H85&gt;=G85*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A85="","",IF(D85=0,"Check target/activation",IF(C85="Seed","P2 keep (seeding)",IF(H85&gt;=G85,"P2 hero - scale",IF(AND(B85="0→1 validate",F85&lt;50),"Learning - hold until ~50 conversions",IF(H85&gt;=G85*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="J86" s="6">
-        <f>IF(A86="","",IF(D86=0,"Check target/activation",IF(C86="Seed","P2 keep (seeding)",IF(H86&gt;=G86,"P2 hero - scale",IF(H86&gt;=G86*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A86="","",IF(D86=0,"Check target/activation",IF(C86="Seed","P2 keep (seeding)",IF(H86&gt;=G86,"P2 hero - scale",IF(AND(B86="0→1 validate",F86&lt;50),"Learning - hold until ~50 conversions",IF(H86&gt;=G86*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
         <v/>
       </c>
       <c r="J87" s="6">
-        <f>IF(A87="","",IF(D87=0,"Check target/activation",IF(C87="Seed","P2 keep (seeding)",IF(H87&gt;=G87,"P2 hero - scale",IF(H87&gt;=G87*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A87="","",IF(D87=0,"Check target/activation",IF(C87="Seed","P2 keep (seeding)",IF(H87&gt;=G87,"P2 hero - scale",IF(AND(B87="0→1 validate",F87&lt;50),"Learning - hold until ~50 conversions",IF(H87&gt;=G87*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2028,7 +2028,7 @@
         <v/>
       </c>
       <c r="J88" s="6">
-        <f>IF(A88="","",IF(D88=0,"Check target/activation",IF(C88="Seed","P2 keep (seeding)",IF(H88&gt;=G88,"P2 hero - scale",IF(H88&gt;=G88*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A88="","",IF(D88=0,"Check target/activation",IF(C88="Seed","P2 keep (seeding)",IF(H88&gt;=G88,"P2 hero - scale",IF(AND(B88="0→1 validate",F88&lt;50),"Learning - hold until ~50 conversions",IF(H88&gt;=G88*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
         <v/>
       </c>
       <c r="J89" s="6">
-        <f>IF(A89="","",IF(D89=0,"Check target/activation",IF(C89="Seed","P2 keep (seeding)",IF(H89&gt;=G89,"P2 hero - scale",IF(H89&gt;=G89*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A89="","",IF(D89=0,"Check target/activation",IF(C89="Seed","P2 keep (seeding)",IF(H89&gt;=G89,"P2 hero - scale",IF(AND(B89="0→1 validate",F89&lt;50),"Learning - hold until ~50 conversions",IF(H89&gt;=G89*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
         <v/>
       </c>
       <c r="J90" s="6">
-        <f>IF(A90="","",IF(D90=0,"Check target/activation",IF(C90="Seed","P2 keep (seeding)",IF(H90&gt;=G90,"P2 hero - scale",IF(H90&gt;=G90*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A90="","",IF(D90=0,"Check target/activation",IF(C90="Seed","P2 keep (seeding)",IF(H90&gt;=G90,"P2 hero - scale",IF(AND(B90="0→1 validate",F90&lt;50),"Learning - hold until ~50 conversions",IF(H90&gt;=G90*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
         <v/>
       </c>
       <c r="J91" s="6">
-        <f>IF(A91="","",IF(D91=0,"Check target/activation",IF(C91="Seed","P2 keep (seeding)",IF(H91&gt;=G91,"P2 hero - scale",IF(H91&gt;=G91*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A91="","",IF(D91=0,"Check target/activation",IF(C91="Seed","P2 keep (seeding)",IF(H91&gt;=G91,"P2 hero - scale",IF(AND(B91="0→1 validate",F91&lt;50),"Learning - hold until ~50 conversions",IF(H91&gt;=G91*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
         <v/>
       </c>
       <c r="J92" s="6">
-        <f>IF(A92="","",IF(D92=0,"Check target/activation",IF(C92="Seed","P2 keep (seeding)",IF(H92&gt;=G92,"P2 hero - scale",IF(H92&gt;=G92*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A92="","",IF(D92=0,"Check target/activation",IF(C92="Seed","P2 keep (seeding)",IF(H92&gt;=G92,"P2 hero - scale",IF(AND(B92="0→1 validate",F92&lt;50),"Learning - hold until ~50 conversions",IF(H92&gt;=G92*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2113,7 +2113,7 @@
         <v/>
       </c>
       <c r="J93" s="6">
-        <f>IF(A93="","",IF(D93=0,"Check target/activation",IF(C93="Seed","P2 keep (seeding)",IF(H93&gt;=G93,"P2 hero - scale",IF(H93&gt;=G93*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A93="","",IF(D93=0,"Check target/activation",IF(C93="Seed","P2 keep (seeding)",IF(H93&gt;=G93,"P2 hero - scale",IF(AND(B93="0→1 validate",F93&lt;50),"Learning - hold until ~50 conversions",IF(H93&gt;=G93*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
         <v/>
       </c>
       <c r="J94" s="6">
-        <f>IF(A94="","",IF(D94=0,"Check target/activation",IF(C94="Seed","P2 keep (seeding)",IF(H94&gt;=G94,"P2 hero - scale",IF(H94&gt;=G94*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A94="","",IF(D94=0,"Check target/activation",IF(C94="Seed","P2 keep (seeding)",IF(H94&gt;=G94,"P2 hero - scale",IF(AND(B94="0→1 validate",F94&lt;50),"Learning - hold until ~50 conversions",IF(H94&gt;=G94*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
         <v/>
       </c>
       <c r="J95" s="6">
-        <f>IF(A95="","",IF(D95=0,"Check target/activation",IF(C95="Seed","P2 keep (seeding)",IF(H95&gt;=G95,"P2 hero - scale",IF(H95&gt;=G95*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A95="","",IF(D95=0,"Check target/activation",IF(C95="Seed","P2 keep (seeding)",IF(H95&gt;=G95,"P2 hero - scale",IF(AND(B95="0→1 validate",F95&lt;50),"Learning - hold until ~50 conversions",IF(H95&gt;=G95*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
         <v/>
       </c>
       <c r="J96" s="6">
-        <f>IF(A96="","",IF(D96=0,"Check target/activation",IF(C96="Seed","P2 keep (seeding)",IF(H96&gt;=G96,"P2 hero - scale",IF(H96&gt;=G96*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A96="","",IF(D96=0,"Check target/activation",IF(C96="Seed","P2 keep (seeding)",IF(H96&gt;=G96,"P2 hero - scale",IF(AND(B96="0→1 validate",F96&lt;50),"Learning - hold until ~50 conversions",IF(H96&gt;=G96*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="J97" s="6">
-        <f>IF(A97="","",IF(D97=0,"Check target/activation",IF(C97="Seed","P2 keep (seeding)",IF(H97&gt;=G97,"P2 hero - scale",IF(H97&gt;=G97*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A97="","",IF(D97=0,"Check target/activation",IF(C97="Seed","P2 keep (seeding)",IF(H97&gt;=G97,"P2 hero - scale",IF(AND(B97="0→1 validate",F97&lt;50),"Learning - hold until ~50 conversions",IF(H97&gt;=G97*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2198,7 +2198,7 @@
         <v/>
       </c>
       <c r="J98" s="6">
-        <f>IF(A98="","",IF(D98=0,"Check target/activation",IF(C98="Seed","P2 keep (seeding)",IF(H98&gt;=G98,"P2 hero - scale",IF(H98&gt;=G98*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A98="","",IF(D98=0,"Check target/activation",IF(C98="Seed","P2 keep (seeding)",IF(H98&gt;=G98,"P2 hero - scale",IF(AND(B98="0→1 validate",F98&lt;50),"Learning - hold until ~50 conversions",IF(H98&gt;=G98*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2215,7 +2215,7 @@
         <v/>
       </c>
       <c r="J99" s="6">
-        <f>IF(A99="","",IF(D99=0,"Check target/activation",IF(C99="Seed","P2 keep (seeding)",IF(H99&gt;=G99,"P2 hero - scale",IF(H99&gt;=G99*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A99="","",IF(D99=0,"Check target/activation",IF(C99="Seed","P2 keep (seeding)",IF(H99&gt;=G99,"P2 hero - scale",IF(AND(B99="0→1 validate",F99&lt;50),"Learning - hold until ~50 conversions",IF(H99&gt;=G99*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
         <v/>
       </c>
       <c r="J100" s="6">
-        <f>IF(A100="","",IF(D100=0,"Check target/activation",IF(C100="Seed","P2 keep (seeding)",IF(H100&gt;=G100,"P2 hero - scale",IF(H100&gt;=G100*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A100="","",IF(D100=0,"Check target/activation",IF(C100="Seed","P2 keep (seeding)",IF(H100&gt;=G100,"P2 hero - scale",IF(AND(B100="0→1 validate",F100&lt;50),"Learning - hold until ~50 conversions",IF(H100&gt;=G100*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
         <v/>
       </c>
       <c r="J101" s="6">
-        <f>IF(A101="","",IF(D101=0,"Check target/activation",IF(C101="Seed","P2 keep (seeding)",IF(H101&gt;=G101,"P2 hero - scale",IF(H101&gt;=G101*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A101="","",IF(D101=0,"Check target/activation",IF(C101="Seed","P2 keep (seeding)",IF(H101&gt;=G101,"P2 hero - scale",IF(AND(B101="0→1 validate",F101&lt;50),"Learning - hold until ~50 conversions",IF(H101&gt;=G101*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
         <v/>
       </c>
       <c r="J102" s="6">
-        <f>IF(A102="","",IF(D102=0,"Check target/activation",IF(C102="Seed","P2 keep (seeding)",IF(H102&gt;=G102,"P2 hero - scale",IF(H102&gt;=G102*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A102="","",IF(D102=0,"Check target/activation",IF(C102="Seed","P2 keep (seeding)",IF(H102&gt;=G102,"P2 hero - scale",IF(AND(B102="0→1 validate",F102&lt;50),"Learning - hold until ~50 conversions",IF(H102&gt;=G102*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2283,7 +2283,7 @@
         <v/>
       </c>
       <c r="J103" s="6">
-        <f>IF(A103="","",IF(D103=0,"Check target/activation",IF(C103="Seed","P2 keep (seeding)",IF(H103&gt;=G103,"P2 hero - scale",IF(H103&gt;=G103*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A103="","",IF(D103=0,"Check target/activation",IF(C103="Seed","P2 keep (seeding)",IF(H103&gt;=G103,"P2 hero - scale",IF(AND(B103="0→1 validate",F103&lt;50),"Learning - hold until ~50 conversions",IF(H103&gt;=G103*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
         <v/>
       </c>
       <c r="J104" s="6">
-        <f>IF(A104="","",IF(D104=0,"Check target/activation",IF(C104="Seed","P2 keep (seeding)",IF(H104&gt;=G104,"P2 hero - scale",IF(H104&gt;=G104*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A104="","",IF(D104=0,"Check target/activation",IF(C104="Seed","P2 keep (seeding)",IF(H104&gt;=G104,"P2 hero - scale",IF(AND(B104="0→1 validate",F104&lt;50),"Learning - hold until ~50 conversions",IF(H104&gt;=G104*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
         <v/>
       </c>
       <c r="J105" s="6">
-        <f>IF(A105="","",IF(D105=0,"Check target/activation",IF(C105="Seed","P2 keep (seeding)",IF(H105&gt;=G105,"P2 hero - scale",IF(H105&gt;=G105*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A105="","",IF(D105=0,"Check target/activation",IF(C105="Seed","P2 keep (seeding)",IF(H105&gt;=G105,"P2 hero - scale",IF(AND(B105="0→1 validate",F105&lt;50),"Learning - hold until ~50 conversions",IF(H105&gt;=G105*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
         <v/>
       </c>
       <c r="J106" s="6">
-        <f>IF(A106="","",IF(D106=0,"Check target/activation",IF(C106="Seed","P2 keep (seeding)",IF(H106&gt;=G106,"P2 hero - scale",IF(H106&gt;=G106*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A106="","",IF(D106=0,"Check target/activation",IF(C106="Seed","P2 keep (seeding)",IF(H106&gt;=G106,"P2 hero - scale",IF(AND(B106="0→1 validate",F106&lt;50),"Learning - hold until ~50 conversions",IF(H106&gt;=G106*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
         <v/>
       </c>
       <c r="J107" s="6">
-        <f>IF(A107="","",IF(D107=0,"Check target/activation",IF(C107="Seed","P2 keep (seeding)",IF(H107&gt;=G107,"P2 hero - scale",IF(H107&gt;=G107*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A107="","",IF(D107=0,"Check target/activation",IF(C107="Seed","P2 keep (seeding)",IF(H107&gt;=G107,"P2 hero - scale",IF(AND(B107="0→1 validate",F107&lt;50),"Learning - hold until ~50 conversions",IF(H107&gt;=G107*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2368,7 +2368,7 @@
         <v/>
       </c>
       <c r="J108" s="6">
-        <f>IF(A108="","",IF(D108=0,"Check target/activation",IF(C108="Seed","P2 keep (seeding)",IF(H108&gt;=G108,"P2 hero - scale",IF(H108&gt;=G108*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A108="","",IF(D108=0,"Check target/activation",IF(C108="Seed","P2 keep (seeding)",IF(H108&gt;=G108,"P2 hero - scale",IF(AND(B108="0→1 validate",F108&lt;50),"Learning - hold until ~50 conversions",IF(H108&gt;=G108*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
         <v/>
       </c>
       <c r="J109" s="6">
-        <f>IF(A109="","",IF(D109=0,"Check target/activation",IF(C109="Seed","P2 keep (seeding)",IF(H109&gt;=G109,"P2 hero - scale",IF(H109&gt;=G109*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A109="","",IF(D109=0,"Check target/activation",IF(C109="Seed","P2 keep (seeding)",IF(H109&gt;=G109,"P2 hero - scale",IF(AND(B109="0→1 validate",F109&lt;50),"Learning - hold until ~50 conversions",IF(H109&gt;=G109*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
         <v/>
       </c>
       <c r="J110" s="6">
-        <f>IF(A110="","",IF(D110=0,"Check target/activation",IF(C110="Seed","P2 keep (seeding)",IF(H110&gt;=G110,"P2 hero - scale",IF(H110&gt;=G110*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A110="","",IF(D110=0,"Check target/activation",IF(C110="Seed","P2 keep (seeding)",IF(H110&gt;=G110,"P2 hero - scale",IF(AND(B110="0→1 validate",F110&lt;50),"Learning - hold until ~50 conversions",IF(H110&gt;=G110*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
         <v/>
       </c>
       <c r="J111" s="6">
-        <f>IF(A111="","",IF(D111=0,"Check target/activation",IF(C111="Seed","P2 keep (seeding)",IF(H111&gt;=G111,"P2 hero - scale",IF(H111&gt;=G111*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A111="","",IF(D111=0,"Check target/activation",IF(C111="Seed","P2 keep (seeding)",IF(H111&gt;=G111,"P2 hero - scale",IF(AND(B111="0→1 validate",F111&lt;50),"Learning - hold until ~50 conversions",IF(H111&gt;=G111*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
         <v/>
       </c>
       <c r="J112" s="6">
-        <f>IF(A112="","",IF(D112=0,"Check target/activation",IF(C112="Seed","P2 keep (seeding)",IF(H112&gt;=G112,"P2 hero - scale",IF(H112&gt;=G112*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A112="","",IF(D112=0,"Check target/activation",IF(C112="Seed","P2 keep (seeding)",IF(H112&gt;=G112,"P2 hero - scale",IF(AND(B112="0→1 validate",F112&lt;50),"Learning - hold until ~50 conversions",IF(H112&gt;=G112*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2453,7 +2453,7 @@
         <v/>
       </c>
       <c r="J113" s="6">
-        <f>IF(A113="","",IF(D113=0,"Check target/activation",IF(C113="Seed","P2 keep (seeding)",IF(H113&gt;=G113,"P2 hero - scale",IF(H113&gt;=G113*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A113="","",IF(D113=0,"Check target/activation",IF(C113="Seed","P2 keep (seeding)",IF(H113&gt;=G113,"P2 hero - scale",IF(AND(B113="0→1 validate",F113&lt;50),"Learning - hold until ~50 conversions",IF(H113&gt;=G113*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
         <v/>
       </c>
       <c r="J114" s="6">
-        <f>IF(A114="","",IF(D114=0,"Check target/activation",IF(C114="Seed","P2 keep (seeding)",IF(H114&gt;=G114,"P2 hero - scale",IF(H114&gt;=G114*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A114="","",IF(D114=0,"Check target/activation",IF(C114="Seed","P2 keep (seeding)",IF(H114&gt;=G114,"P2 hero - scale",IF(AND(B114="0→1 validate",F114&lt;50),"Learning - hold until ~50 conversions",IF(H114&gt;=G114*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2487,7 +2487,7 @@
         <v/>
       </c>
       <c r="J115" s="6">
-        <f>IF(A115="","",IF(D115=0,"Check target/activation",IF(C115="Seed","P2 keep (seeding)",IF(H115&gt;=G115,"P2 hero - scale",IF(H115&gt;=G115*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A115="","",IF(D115=0,"Check target/activation",IF(C115="Seed","P2 keep (seeding)",IF(H115&gt;=G115,"P2 hero - scale",IF(AND(B115="0→1 validate",F115&lt;50),"Learning - hold until ~50 conversions",IF(H115&gt;=G115*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
         <v/>
       </c>
       <c r="J116" s="6">
-        <f>IF(A116="","",IF(D116=0,"Check target/activation",IF(C116="Seed","P2 keep (seeding)",IF(H116&gt;=G116,"P2 hero - scale",IF(H116&gt;=G116*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A116="","",IF(D116=0,"Check target/activation",IF(C116="Seed","P2 keep (seeding)",IF(H116&gt;=G116,"P2 hero - scale",IF(AND(B116="0→1 validate",F116&lt;50),"Learning - hold until ~50 conversions",IF(H116&gt;=G116*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
         <v/>
       </c>
       <c r="J117" s="6">
-        <f>IF(A117="","",IF(D117=0,"Check target/activation",IF(C117="Seed","P2 keep (seeding)",IF(H117&gt;=G117,"P2 hero - scale",IF(H117&gt;=G117*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A117="","",IF(D117=0,"Check target/activation",IF(C117="Seed","P2 keep (seeding)",IF(H117&gt;=G117,"P2 hero - scale",IF(AND(B117="0→1 validate",F117&lt;50),"Learning - hold until ~50 conversions",IF(H117&gt;=G117*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2538,7 +2538,7 @@
         <v/>
       </c>
       <c r="J118" s="6">
-        <f>IF(A118="","",IF(D118=0,"Check target/activation",IF(C118="Seed","P2 keep (seeding)",IF(H118&gt;=G118,"P2 hero - scale",IF(H118&gt;=G118*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A118="","",IF(D118=0,"Check target/activation",IF(C118="Seed","P2 keep (seeding)",IF(H118&gt;=G118,"P2 hero - scale",IF(AND(B118="0→1 validate",F118&lt;50),"Learning - hold until ~50 conversions",IF(H118&gt;=G118*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
         <v/>
       </c>
       <c r="J119" s="6">
-        <f>IF(A119="","",IF(D119=0,"Check target/activation",IF(C119="Seed","P2 keep (seeding)",IF(H119&gt;=G119,"P2 hero - scale",IF(H119&gt;=G119*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A119="","",IF(D119=0,"Check target/activation",IF(C119="Seed","P2 keep (seeding)",IF(H119&gt;=G119,"P2 hero - scale",IF(AND(B119="0→1 validate",F119&lt;50),"Learning - hold until ~50 conversions",IF(H119&gt;=G119*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
         <v/>
       </c>
       <c r="J120" s="6">
-        <f>IF(A120="","",IF(D120=0,"Check target/activation",IF(C120="Seed","P2 keep (seeding)",IF(H120&gt;=G120,"P2 hero - scale",IF(H120&gt;=G120*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A120="","",IF(D120=0,"Check target/activation",IF(C120="Seed","P2 keep (seeding)",IF(H120&gt;=G120,"P2 hero - scale",IF(AND(B120="0→1 validate",F120&lt;50),"Learning - hold until ~50 conversions",IF(H120&gt;=G120*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
         <v/>
       </c>
       <c r="J121" s="6">
-        <f>IF(A121="","",IF(D121=0,"Check target/activation",IF(C121="Seed","P2 keep (seeding)",IF(H121&gt;=G121,"P2 hero - scale",IF(H121&gt;=G121*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A121="","",IF(D121=0,"Check target/activation",IF(C121="Seed","P2 keep (seeding)",IF(H121&gt;=G121,"P2 hero - scale",IF(AND(B121="0→1 validate",F121&lt;50),"Learning - hold until ~50 conversions",IF(H121&gt;=G121*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2606,7 +2606,7 @@
         <v/>
       </c>
       <c r="J122" s="6">
-        <f>IF(A122="","",IF(D122=0,"Check target/activation",IF(C122="Seed","P2 keep (seeding)",IF(H122&gt;=G122,"P2 hero - scale",IF(H122&gt;=G122*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A122="","",IF(D122=0,"Check target/activation",IF(C122="Seed","P2 keep (seeding)",IF(H122&gt;=G122,"P2 hero - scale",IF(AND(B122="0→1 validate",F122&lt;50),"Learning - hold until ~50 conversions",IF(H122&gt;=G122*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
         <v/>
       </c>
       <c r="J123" s="6">
-        <f>IF(A123="","",IF(D123=0,"Check target/activation",IF(C123="Seed","P2 keep (seeding)",IF(H123&gt;=G123,"P2 hero - scale",IF(H123&gt;=G123*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A123="","",IF(D123=0,"Check target/activation",IF(C123="Seed","P2 keep (seeding)",IF(H123&gt;=G123,"P2 hero - scale",IF(AND(B123="0→1 validate",F123&lt;50),"Learning - hold until ~50 conversions",IF(H123&gt;=G123*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2640,7 +2640,7 @@
         <v/>
       </c>
       <c r="J124" s="6">
-        <f>IF(A124="","",IF(D124=0,"Check target/activation",IF(C124="Seed","P2 keep (seeding)",IF(H124&gt;=G124,"P2 hero - scale",IF(H124&gt;=G124*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A124="","",IF(D124=0,"Check target/activation",IF(C124="Seed","P2 keep (seeding)",IF(H124&gt;=G124,"P2 hero - scale",IF(AND(B124="0→1 validate",F124&lt;50),"Learning - hold until ~50 conversions",IF(H124&gt;=G124*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
         <v/>
       </c>
       <c r="J125" s="6">
-        <f>IF(A125="","",IF(D125=0,"Check target/activation",IF(C125="Seed","P2 keep (seeding)",IF(H125&gt;=G125,"P2 hero - scale",IF(H125&gt;=G125*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A125="","",IF(D125=0,"Check target/activation",IF(C125="Seed","P2 keep (seeding)",IF(H125&gt;=G125,"P2 hero - scale",IF(AND(B125="0→1 validate",F125&lt;50),"Learning - hold until ~50 conversions",IF(H125&gt;=G125*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
         <v/>
       </c>
       <c r="J126" s="6">
-        <f>IF(A126="","",IF(D126=0,"Check target/activation",IF(C126="Seed","P2 keep (seeding)",IF(H126&gt;=G126,"P2 hero - scale",IF(H126&gt;=G126*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A126="","",IF(D126=0,"Check target/activation",IF(C126="Seed","P2 keep (seeding)",IF(H126&gt;=G126,"P2 hero - scale",IF(AND(B126="0→1 validate",F126&lt;50),"Learning - hold until ~50 conversions",IF(H126&gt;=G126*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
         <v/>
       </c>
       <c r="J127" s="6">
-        <f>IF(A127="","",IF(D127=0,"Check target/activation",IF(C127="Seed","P2 keep (seeding)",IF(H127&gt;=G127,"P2 hero - scale",IF(H127&gt;=G127*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A127="","",IF(D127=0,"Check target/activation",IF(C127="Seed","P2 keep (seeding)",IF(H127&gt;=G127,"P2 hero - scale",IF(AND(B127="0→1 validate",F127&lt;50),"Learning - hold until ~50 conversions",IF(H127&gt;=G127*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
         <v/>
       </c>
       <c r="J128" s="6">
-        <f>IF(A128="","",IF(D128=0,"Check target/activation",IF(C128="Seed","P2 keep (seeding)",IF(H128&gt;=G128,"P2 hero - scale",IF(H128&gt;=G128*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A128="","",IF(D128=0,"Check target/activation",IF(C128="Seed","P2 keep (seeding)",IF(H128&gt;=G128,"P2 hero - scale",IF(AND(B128="0→1 validate",F128&lt;50),"Learning - hold until ~50 conversions",IF(H128&gt;=G128*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2725,7 +2725,7 @@
         <v/>
       </c>
       <c r="J129" s="6">
-        <f>IF(A129="","",IF(D129=0,"Check target/activation",IF(C129="Seed","P2 keep (seeding)",IF(H129&gt;=G129,"P2 hero - scale",IF(H129&gt;=G129*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A129="","",IF(D129=0,"Check target/activation",IF(C129="Seed","P2 keep (seeding)",IF(H129&gt;=G129,"P2 hero - scale",IF(AND(B129="0→1 validate",F129&lt;50),"Learning - hold until ~50 conversions",IF(H129&gt;=G129*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
         <v/>
       </c>
       <c r="J130" s="6">
-        <f>IF(A130="","",IF(D130=0,"Check target/activation",IF(C130="Seed","P2 keep (seeding)",IF(H130&gt;=G130,"P2 hero - scale",IF(H130&gt;=G130*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A130="","",IF(D130=0,"Check target/activation",IF(C130="Seed","P2 keep (seeding)",IF(H130&gt;=G130,"P2 hero - scale",IF(AND(B130="0→1 validate",F130&lt;50),"Learning - hold until ~50 conversions",IF(H130&gt;=G130*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
         <v/>
       </c>
       <c r="J131" s="6">
-        <f>IF(A131="","",IF(D131=0,"Check target/activation",IF(C131="Seed","P2 keep (seeding)",IF(H131&gt;=G131,"P2 hero - scale",IF(H131&gt;=G131*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A131="","",IF(D131=0,"Check target/activation",IF(C131="Seed","P2 keep (seeding)",IF(H131&gt;=G131,"P2 hero - scale",IF(AND(B131="0→1 validate",F131&lt;50),"Learning - hold until ~50 conversions",IF(H131&gt;=G131*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2776,7 +2776,7 @@
         <v/>
       </c>
       <c r="J132" s="6">
-        <f>IF(A132="","",IF(D132=0,"Check target/activation",IF(C132="Seed","P2 keep (seeding)",IF(H132&gt;=G132,"P2 hero - scale",IF(H132&gt;=G132*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A132="","",IF(D132=0,"Check target/activation",IF(C132="Seed","P2 keep (seeding)",IF(H132&gt;=G132,"P2 hero - scale",IF(AND(B132="0→1 validate",F132&lt;50),"Learning - hold until ~50 conversions",IF(H132&gt;=G132*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2793,7 +2793,7 @@
         <v/>
       </c>
       <c r="J133" s="6">
-        <f>IF(A133="","",IF(D133=0,"Check target/activation",IF(C133="Seed","P2 keep (seeding)",IF(H133&gt;=G133,"P2 hero - scale",IF(H133&gt;=G133*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A133="","",IF(D133=0,"Check target/activation",IF(C133="Seed","P2 keep (seeding)",IF(H133&gt;=G133,"P2 hero - scale",IF(AND(B133="0→1 validate",F133&lt;50),"Learning - hold until ~50 conversions",IF(H133&gt;=G133*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
         <v/>
       </c>
       <c r="J134" s="6">
-        <f>IF(A134="","",IF(D134=0,"Check target/activation",IF(C134="Seed","P2 keep (seeding)",IF(H134&gt;=G134,"P2 hero - scale",IF(H134&gt;=G134*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A134="","",IF(D134=0,"Check target/activation",IF(C134="Seed","P2 keep (seeding)",IF(H134&gt;=G134,"P2 hero - scale",IF(AND(B134="0→1 validate",F134&lt;50),"Learning - hold until ~50 conversions",IF(H134&gt;=G134*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2827,7 +2827,7 @@
         <v/>
       </c>
       <c r="J135" s="6">
-        <f>IF(A135="","",IF(D135=0,"Check target/activation",IF(C135="Seed","P2 keep (seeding)",IF(H135&gt;=G135,"P2 hero - scale",IF(H135&gt;=G135*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A135="","",IF(D135=0,"Check target/activation",IF(C135="Seed","P2 keep (seeding)",IF(H135&gt;=G135,"P2 hero - scale",IF(AND(B135="0→1 validate",F135&lt;50),"Learning - hold until ~50 conversions",IF(H135&gt;=G135*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
         <v/>
       </c>
       <c r="J136" s="6">
-        <f>IF(A136="","",IF(D136=0,"Check target/activation",IF(C136="Seed","P2 keep (seeding)",IF(H136&gt;=G136,"P2 hero - scale",IF(H136&gt;=G136*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A136="","",IF(D136=0,"Check target/activation",IF(C136="Seed","P2 keep (seeding)",IF(H136&gt;=G136,"P2 hero - scale",IF(AND(B136="0→1 validate",F136&lt;50),"Learning - hold until ~50 conversions",IF(H136&gt;=G136*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
         <v/>
       </c>
       <c r="J137" s="6">
-        <f>IF(A137="","",IF(D137=0,"Check target/activation",IF(C137="Seed","P2 keep (seeding)",IF(H137&gt;=G137,"P2 hero - scale",IF(H137&gt;=G137*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A137="","",IF(D137=0,"Check target/activation",IF(C137="Seed","P2 keep (seeding)",IF(H137&gt;=G137,"P2 hero - scale",IF(AND(B137="0→1 validate",F137&lt;50),"Learning - hold until ~50 conversions",IF(H137&gt;=G137*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2878,7 +2878,7 @@
         <v/>
       </c>
       <c r="J138" s="6">
-        <f>IF(A138="","",IF(D138=0,"Check target/activation",IF(C138="Seed","P2 keep (seeding)",IF(H138&gt;=G138,"P2 hero - scale",IF(H138&gt;=G138*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A138="","",IF(D138=0,"Check target/activation",IF(C138="Seed","P2 keep (seeding)",IF(H138&gt;=G138,"P2 hero - scale",IF(AND(B138="0→1 validate",F138&lt;50),"Learning - hold until ~50 conversions",IF(H138&gt;=G138*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
         <v/>
       </c>
       <c r="J139" s="6">
-        <f>IF(A139="","",IF(D139=0,"Check target/activation",IF(C139="Seed","P2 keep (seeding)",IF(H139&gt;=G139,"P2 hero - scale",IF(H139&gt;=G139*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A139="","",IF(D139=0,"Check target/activation",IF(C139="Seed","P2 keep (seeding)",IF(H139&gt;=G139,"P2 hero - scale",IF(AND(B139="0→1 validate",F139&lt;50),"Learning - hold until ~50 conversions",IF(H139&gt;=G139*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
         <v/>
       </c>
       <c r="J140" s="6">
-        <f>IF(A140="","",IF(D140=0,"Check target/activation",IF(C140="Seed","P2 keep (seeding)",IF(H140&gt;=G140,"P2 hero - scale",IF(H140&gt;=G140*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A140="","",IF(D140=0,"Check target/activation",IF(C140="Seed","P2 keep (seeding)",IF(H140&gt;=G140,"P2 hero - scale",IF(AND(B140="0→1 validate",F140&lt;50),"Learning - hold until ~50 conversions",IF(H140&gt;=G140*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
         <v/>
       </c>
       <c r="J141" s="6">
-        <f>IF(A141="","",IF(D141=0,"Check target/activation",IF(C141="Seed","P2 keep (seeding)",IF(H141&gt;=G141,"P2 hero - scale",IF(H141&gt;=G141*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A141="","",IF(D141=0,"Check target/activation",IF(C141="Seed","P2 keep (seeding)",IF(H141&gt;=G141,"P2 hero - scale",IF(AND(B141="0→1 validate",F141&lt;50),"Learning - hold until ~50 conversions",IF(H141&gt;=G141*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
         <v/>
       </c>
       <c r="J142" s="6">
-        <f>IF(A142="","",IF(D142=0,"Check target/activation",IF(C142="Seed","P2 keep (seeding)",IF(H142&gt;=G142,"P2 hero - scale",IF(H142&gt;=G142*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A142="","",IF(D142=0,"Check target/activation",IF(C142="Seed","P2 keep (seeding)",IF(H142&gt;=G142,"P2 hero - scale",IF(AND(B142="0→1 validate",F142&lt;50),"Learning - hold until ~50 conversions",IF(H142&gt;=G142*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2963,7 +2963,7 @@
         <v/>
       </c>
       <c r="J143" s="6">
-        <f>IF(A143="","",IF(D143=0,"Check target/activation",IF(C143="Seed","P2 keep (seeding)",IF(H143&gt;=G143,"P2 hero - scale",IF(H143&gt;=G143*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A143="","",IF(D143=0,"Check target/activation",IF(C143="Seed","P2 keep (seeding)",IF(H143&gt;=G143,"P2 hero - scale",IF(AND(B143="0→1 validate",F143&lt;50),"Learning - hold until ~50 conversions",IF(H143&gt;=G143*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
         <v/>
       </c>
       <c r="J144" s="6">
-        <f>IF(A144="","",IF(D144=0,"Check target/activation",IF(C144="Seed","P2 keep (seeding)",IF(H144&gt;=G144,"P2 hero - scale",IF(H144&gt;=G144*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A144="","",IF(D144=0,"Check target/activation",IF(C144="Seed","P2 keep (seeding)",IF(H144&gt;=G144,"P2 hero - scale",IF(AND(B144="0→1 validate",F144&lt;50),"Learning - hold until ~50 conversions",IF(H144&gt;=G144*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
         <v/>
       </c>
       <c r="J145" s="6">
-        <f>IF(A145="","",IF(D145=0,"Check target/activation",IF(C145="Seed","P2 keep (seeding)",IF(H145&gt;=G145,"P2 hero - scale",IF(H145&gt;=G145*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A145="","",IF(D145=0,"Check target/activation",IF(C145="Seed","P2 keep (seeding)",IF(H145&gt;=G145,"P2 hero - scale",IF(AND(B145="0→1 validate",F145&lt;50),"Learning - hold until ~50 conversions",IF(H145&gt;=G145*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="J146" s="6">
-        <f>IF(A146="","",IF(D146=0,"Check target/activation",IF(C146="Seed","P2 keep (seeding)",IF(H146&gt;=G146,"P2 hero - scale",IF(H146&gt;=G146*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A146="","",IF(D146=0,"Check target/activation",IF(C146="Seed","P2 keep (seeding)",IF(H146&gt;=G146,"P2 hero - scale",IF(AND(B146="0→1 validate",F146&lt;50),"Learning - hold until ~50 conversions",IF(H146&gt;=G146*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
         <v/>
       </c>
       <c r="J147" s="6">
-        <f>IF(A147="","",IF(D147=0,"Check target/activation",IF(C147="Seed","P2 keep (seeding)",IF(H147&gt;=G147,"P2 hero - scale",IF(H147&gt;=G147*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A147="","",IF(D147=0,"Check target/activation",IF(C147="Seed","P2 keep (seeding)",IF(H147&gt;=G147,"P2 hero - scale",IF(AND(B147="0→1 validate",F147&lt;50),"Learning - hold until ~50 conversions",IF(H147&gt;=G147*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
         <v/>
       </c>
       <c r="J148" s="6">
-        <f>IF(A148="","",IF(D148=0,"Check target/activation",IF(C148="Seed","P2 keep (seeding)",IF(H148&gt;=G148,"P2 hero - scale",IF(H148&gt;=G148*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A148="","",IF(D148=0,"Check target/activation",IF(C148="Seed","P2 keep (seeding)",IF(H148&gt;=G148,"P2 hero - scale",IF(AND(B148="0→1 validate",F148&lt;50),"Learning - hold until ~50 conversions",IF(H148&gt;=G148*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3065,7 +3065,7 @@
         <v/>
       </c>
       <c r="J149" s="6">
-        <f>IF(A149="","",IF(D149=0,"Check target/activation",IF(C149="Seed","P2 keep (seeding)",IF(H149&gt;=G149,"P2 hero - scale",IF(H149&gt;=G149*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A149="","",IF(D149=0,"Check target/activation",IF(C149="Seed","P2 keep (seeding)",IF(H149&gt;=G149,"P2 hero - scale",IF(AND(B149="0→1 validate",F149&lt;50),"Learning - hold until ~50 conversions",IF(H149&gt;=G149*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="J150" s="6">
-        <f>IF(A150="","",IF(D150=0,"Check target/activation",IF(C150="Seed","P2 keep (seeding)",IF(H150&gt;=G150,"P2 hero - scale",IF(H150&gt;=G150*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A150="","",IF(D150=0,"Check target/activation",IF(C150="Seed","P2 keep (seeding)",IF(H150&gt;=G150,"P2 hero - scale",IF(AND(B150="0→1 validate",F150&lt;50),"Learning - hold until ~50 conversions",IF(H150&gt;=G150*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3099,7 +3099,7 @@
         <v/>
       </c>
       <c r="J151" s="6">
-        <f>IF(A151="","",IF(D151=0,"Check target/activation",IF(C151="Seed","P2 keep (seeding)",IF(H151&gt;=G151,"P2 hero - scale",IF(H151&gt;=G151*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A151="","",IF(D151=0,"Check target/activation",IF(C151="Seed","P2 keep (seeding)",IF(H151&gt;=G151,"P2 hero - scale",IF(AND(B151="0→1 validate",F151&lt;50),"Learning - hold until ~50 conversions",IF(H151&gt;=G151*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v/>
       </c>
       <c r="J152" s="6">
-        <f>IF(A152="","",IF(D152=0,"Check target/activation",IF(C152="Seed","P2 keep (seeding)",IF(H152&gt;=G152,"P2 hero - scale",IF(H152&gt;=G152*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A152="","",IF(D152=0,"Check target/activation",IF(C152="Seed","P2 keep (seeding)",IF(H152&gt;=G152,"P2 hero - scale",IF(AND(B152="0→1 validate",F152&lt;50),"Learning - hold until ~50 conversions",IF(H152&gt;=G152*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3133,7 +3133,7 @@
         <v/>
       </c>
       <c r="J153" s="6">
-        <f>IF(A153="","",IF(D153=0,"Check target/activation",IF(C153="Seed","P2 keep (seeding)",IF(H153&gt;=G153,"P2 hero - scale",IF(H153&gt;=G153*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A153="","",IF(D153=0,"Check target/activation",IF(C153="Seed","P2 keep (seeding)",IF(H153&gt;=G153,"P2 hero - scale",IF(AND(B153="0→1 validate",F153&lt;50),"Learning - hold until ~50 conversions",IF(H153&gt;=G153*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3150,7 +3150,7 @@
         <v/>
       </c>
       <c r="J154" s="6">
-        <f>IF(A154="","",IF(D154=0,"Check target/activation",IF(C154="Seed","P2 keep (seeding)",IF(H154&gt;=G154,"P2 hero - scale",IF(H154&gt;=G154*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A154="","",IF(D154=0,"Check target/activation",IF(C154="Seed","P2 keep (seeding)",IF(H154&gt;=G154,"P2 hero - scale",IF(AND(B154="0→1 validate",F154&lt;50),"Learning - hold until ~50 conversions",IF(H154&gt;=G154*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
         <v/>
       </c>
       <c r="J155" s="6">
-        <f>IF(A155="","",IF(D155=0,"Check target/activation",IF(C155="Seed","P2 keep (seeding)",IF(H155&gt;=G155,"P2 hero - scale",IF(H155&gt;=G155*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A155="","",IF(D155=0,"Check target/activation",IF(C155="Seed","P2 keep (seeding)",IF(H155&gt;=G155,"P2 hero - scale",IF(AND(B155="0→1 validate",F155&lt;50),"Learning - hold until ~50 conversions",IF(H155&gt;=G155*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
         <v/>
       </c>
       <c r="J156" s="6">
-        <f>IF(A156="","",IF(D156=0,"Check target/activation",IF(C156="Seed","P2 keep (seeding)",IF(H156&gt;=G156,"P2 hero - scale",IF(H156&gt;=G156*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A156="","",IF(D156=0,"Check target/activation",IF(C156="Seed","P2 keep (seeding)",IF(H156&gt;=G156,"P2 hero - scale",IF(AND(B156="0→1 validate",F156&lt;50),"Learning - hold until ~50 conversions",IF(H156&gt;=G156*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
         <v/>
       </c>
       <c r="J157" s="6">
-        <f>IF(A157="","",IF(D157=0,"Check target/activation",IF(C157="Seed","P2 keep (seeding)",IF(H157&gt;=G157,"P2 hero - scale",IF(H157&gt;=G157*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A157="","",IF(D157=0,"Check target/activation",IF(C157="Seed","P2 keep (seeding)",IF(H157&gt;=G157,"P2 hero - scale",IF(AND(B157="0→1 validate",F157&lt;50),"Learning - hold until ~50 conversions",IF(H157&gt;=G157*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3218,7 +3218,7 @@
         <v/>
       </c>
       <c r="J158" s="6">
-        <f>IF(A158="","",IF(D158=0,"Check target/activation",IF(C158="Seed","P2 keep (seeding)",IF(H158&gt;=G158,"P2 hero - scale",IF(H158&gt;=G158*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A158="","",IF(D158=0,"Check target/activation",IF(C158="Seed","P2 keep (seeding)",IF(H158&gt;=G158,"P2 hero - scale",IF(AND(B158="0→1 validate",F158&lt;50),"Learning - hold until ~50 conversions",IF(H158&gt;=G158*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
         <v/>
       </c>
       <c r="J159" s="6">
-        <f>IF(A159="","",IF(D159=0,"Check target/activation",IF(C159="Seed","P2 keep (seeding)",IF(H159&gt;=G159,"P2 hero - scale",IF(H159&gt;=G159*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A159="","",IF(D159=0,"Check target/activation",IF(C159="Seed","P2 keep (seeding)",IF(H159&gt;=G159,"P2 hero - scale",IF(AND(B159="0→1 validate",F159&lt;50),"Learning - hold until ~50 conversions",IF(H159&gt;=G159*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
         <v/>
       </c>
       <c r="J160" s="6">
-        <f>IF(A160="","",IF(D160=0,"Check target/activation",IF(C160="Seed","P2 keep (seeding)",IF(H160&gt;=G160,"P2 hero - scale",IF(H160&gt;=G160*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A160="","",IF(D160=0,"Check target/activation",IF(C160="Seed","P2 keep (seeding)",IF(H160&gt;=G160,"P2 hero - scale",IF(AND(B160="0→1 validate",F160&lt;50),"Learning - hold until ~50 conversions",IF(H160&gt;=G160*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3269,7 +3269,7 @@
         <v/>
       </c>
       <c r="J161" s="6">
-        <f>IF(A161="","",IF(D161=0,"Check target/activation",IF(C161="Seed","P2 keep (seeding)",IF(H161&gt;=G161,"P2 hero - scale",IF(H161&gt;=G161*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A161="","",IF(D161=0,"Check target/activation",IF(C161="Seed","P2 keep (seeding)",IF(H161&gt;=G161,"P2 hero - scale",IF(AND(B161="0→1 validate",F161&lt;50),"Learning - hold until ~50 conversions",IF(H161&gt;=G161*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3286,7 +3286,7 @@
         <v/>
       </c>
       <c r="J162" s="6">
-        <f>IF(A162="","",IF(D162=0,"Check target/activation",IF(C162="Seed","P2 keep (seeding)",IF(H162&gt;=G162,"P2 hero - scale",IF(H162&gt;=G162*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A162="","",IF(D162=0,"Check target/activation",IF(C162="Seed","P2 keep (seeding)",IF(H162&gt;=G162,"P2 hero - scale",IF(AND(B162="0→1 validate",F162&lt;50),"Learning - hold until ~50 conversions",IF(H162&gt;=G162*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
         <v/>
       </c>
       <c r="J163" s="6">
-        <f>IF(A163="","",IF(D163=0,"Check target/activation",IF(C163="Seed","P2 keep (seeding)",IF(H163&gt;=G163,"P2 hero - scale",IF(H163&gt;=G163*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A163="","",IF(D163=0,"Check target/activation",IF(C163="Seed","P2 keep (seeding)",IF(H163&gt;=G163,"P2 hero - scale",IF(AND(B163="0→1 validate",F163&lt;50),"Learning - hold until ~50 conversions",IF(H163&gt;=G163*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3320,7 +3320,7 @@
         <v/>
       </c>
       <c r="J164" s="6">
-        <f>IF(A164="","",IF(D164=0,"Check target/activation",IF(C164="Seed","P2 keep (seeding)",IF(H164&gt;=G164,"P2 hero - scale",IF(H164&gt;=G164*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A164="","",IF(D164=0,"Check target/activation",IF(C164="Seed","P2 keep (seeding)",IF(H164&gt;=G164,"P2 hero - scale",IF(AND(B164="0→1 validate",F164&lt;50),"Learning - hold until ~50 conversions",IF(H164&gt;=G164*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
         <v/>
       </c>
       <c r="J165" s="6">
-        <f>IF(A165="","",IF(D165=0,"Check target/activation",IF(C165="Seed","P2 keep (seeding)",IF(H165&gt;=G165,"P2 hero - scale",IF(H165&gt;=G165*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A165="","",IF(D165=0,"Check target/activation",IF(C165="Seed","P2 keep (seeding)",IF(H165&gt;=G165,"P2 hero - scale",IF(AND(B165="0→1 validate",F165&lt;50),"Learning - hold until ~50 conversions",IF(H165&gt;=G165*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
         <v/>
       </c>
       <c r="J166" s="6">
-        <f>IF(A166="","",IF(D166=0,"Check target/activation",IF(C166="Seed","P2 keep (seeding)",IF(H166&gt;=G166,"P2 hero - scale",IF(H166&gt;=G166*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A166="","",IF(D166=0,"Check target/activation",IF(C166="Seed","P2 keep (seeding)",IF(H166&gt;=G166,"P2 hero - scale",IF(AND(B166="0→1 validate",F166&lt;50),"Learning - hold until ~50 conversions",IF(H166&gt;=G166*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
         <v/>
       </c>
       <c r="J167" s="6">
-        <f>IF(A167="","",IF(D167=0,"Check target/activation",IF(C167="Seed","P2 keep (seeding)",IF(H167&gt;=G167,"P2 hero - scale",IF(H167&gt;=G167*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A167="","",IF(D167=0,"Check target/activation",IF(C167="Seed","P2 keep (seeding)",IF(H167&gt;=G167,"P2 hero - scale",IF(AND(B167="0→1 validate",F167&lt;50),"Learning - hold until ~50 conversions",IF(H167&gt;=G167*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
         <v/>
       </c>
       <c r="J168" s="6">
-        <f>IF(A168="","",IF(D168=0,"Check target/activation",IF(C168="Seed","P2 keep (seeding)",IF(H168&gt;=G168,"P2 hero - scale",IF(H168&gt;=G168*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A168="","",IF(D168=0,"Check target/activation",IF(C168="Seed","P2 keep (seeding)",IF(H168&gt;=G168,"P2 hero - scale",IF(AND(B168="0→1 validate",F168&lt;50),"Learning - hold until ~50 conversions",IF(H168&gt;=G168*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3405,7 +3405,7 @@
         <v/>
       </c>
       <c r="J169" s="6">
-        <f>IF(A169="","",IF(D169=0,"Check target/activation",IF(C169="Seed","P2 keep (seeding)",IF(H169&gt;=G169,"P2 hero - scale",IF(H169&gt;=G169*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A169="","",IF(D169=0,"Check target/activation",IF(C169="Seed","P2 keep (seeding)",IF(H169&gt;=G169,"P2 hero - scale",IF(AND(B169="0→1 validate",F169&lt;50),"Learning - hold until ~50 conversions",IF(H169&gt;=G169*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
         <v/>
       </c>
       <c r="J170" s="6">
-        <f>IF(A170="","",IF(D170=0,"Check target/activation",IF(C170="Seed","P2 keep (seeding)",IF(H170&gt;=G170,"P2 hero - scale",IF(H170&gt;=G170*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A170="","",IF(D170=0,"Check target/activation",IF(C170="Seed","P2 keep (seeding)",IF(H170&gt;=G170,"P2 hero - scale",IF(AND(B170="0→1 validate",F170&lt;50),"Learning - hold until ~50 conversions",IF(H170&gt;=G170*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3439,7 +3439,7 @@
         <v/>
       </c>
       <c r="J171" s="6">
-        <f>IF(A171="","",IF(D171=0,"Check target/activation",IF(C171="Seed","P2 keep (seeding)",IF(H171&gt;=G171,"P2 hero - scale",IF(H171&gt;=G171*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A171="","",IF(D171=0,"Check target/activation",IF(C171="Seed","P2 keep (seeding)",IF(H171&gt;=G171,"P2 hero - scale",IF(AND(B171="0→1 validate",F171&lt;50),"Learning - hold until ~50 conversions",IF(H171&gt;=G171*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3456,7 +3456,7 @@
         <v/>
       </c>
       <c r="J172" s="6">
-        <f>IF(A172="","",IF(D172=0,"Check target/activation",IF(C172="Seed","P2 keep (seeding)",IF(H172&gt;=G172,"P2 hero - scale",IF(H172&gt;=G172*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A172="","",IF(D172=0,"Check target/activation",IF(C172="Seed","P2 keep (seeding)",IF(H172&gt;=G172,"P2 hero - scale",IF(AND(B172="0→1 validate",F172&lt;50),"Learning - hold until ~50 conversions",IF(H172&gt;=G172*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3473,7 +3473,7 @@
         <v/>
       </c>
       <c r="J173" s="6">
-        <f>IF(A173="","",IF(D173=0,"Check target/activation",IF(C173="Seed","P2 keep (seeding)",IF(H173&gt;=G173,"P2 hero - scale",IF(H173&gt;=G173*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A173="","",IF(D173=0,"Check target/activation",IF(C173="Seed","P2 keep (seeding)",IF(H173&gt;=G173,"P2 hero - scale",IF(AND(B173="0→1 validate",F173&lt;50),"Learning - hold until ~50 conversions",IF(H173&gt;=G173*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3490,7 +3490,7 @@
         <v/>
       </c>
       <c r="J174" s="6">
-        <f>IF(A174="","",IF(D174=0,"Check target/activation",IF(C174="Seed","P2 keep (seeding)",IF(H174&gt;=G174,"P2 hero - scale",IF(H174&gt;=G174*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A174="","",IF(D174=0,"Check target/activation",IF(C174="Seed","P2 keep (seeding)",IF(H174&gt;=G174,"P2 hero - scale",IF(AND(B174="0→1 validate",F174&lt;50),"Learning - hold until ~50 conversions",IF(H174&gt;=G174*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3507,7 +3507,7 @@
         <v/>
       </c>
       <c r="J175" s="6">
-        <f>IF(A175="","",IF(D175=0,"Check target/activation",IF(C175="Seed","P2 keep (seeding)",IF(H175&gt;=G175,"P2 hero - scale",IF(H175&gt;=G175*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A175="","",IF(D175=0,"Check target/activation",IF(C175="Seed","P2 keep (seeding)",IF(H175&gt;=G175,"P2 hero - scale",IF(AND(B175="0→1 validate",F175&lt;50),"Learning - hold until ~50 conversions",IF(H175&gt;=G175*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3524,7 +3524,7 @@
         <v/>
       </c>
       <c r="J176" s="6">
-        <f>IF(A176="","",IF(D176=0,"Check target/activation",IF(C176="Seed","P2 keep (seeding)",IF(H176&gt;=G176,"P2 hero - scale",IF(H176&gt;=G176*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A176="","",IF(D176=0,"Check target/activation",IF(C176="Seed","P2 keep (seeding)",IF(H176&gt;=G176,"P2 hero - scale",IF(AND(B176="0→1 validate",F176&lt;50),"Learning - hold until ~50 conversions",IF(H176&gt;=G176*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
         <v/>
       </c>
       <c r="J177" s="6">
-        <f>IF(A177="","",IF(D177=0,"Check target/activation",IF(C177="Seed","P2 keep (seeding)",IF(H177&gt;=G177,"P2 hero - scale",IF(H177&gt;=G177*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A177="","",IF(D177=0,"Check target/activation",IF(C177="Seed","P2 keep (seeding)",IF(H177&gt;=G177,"P2 hero - scale",IF(AND(B177="0→1 validate",F177&lt;50),"Learning - hold until ~50 conversions",IF(H177&gt;=G177*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
         <v/>
       </c>
       <c r="J178" s="6">
-        <f>IF(A178="","",IF(D178=0,"Check target/activation",IF(C178="Seed","P2 keep (seeding)",IF(H178&gt;=G178,"P2 hero - scale",IF(H178&gt;=G178*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A178="","",IF(D178=0,"Check target/activation",IF(C178="Seed","P2 keep (seeding)",IF(H178&gt;=G178,"P2 hero - scale",IF(AND(B178="0→1 validate",F178&lt;50),"Learning - hold until ~50 conversions",IF(H178&gt;=G178*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
         <v/>
       </c>
       <c r="J179" s="6">
-        <f>IF(A179="","",IF(D179=0,"Check target/activation",IF(C179="Seed","P2 keep (seeding)",IF(H179&gt;=G179,"P2 hero - scale",IF(H179&gt;=G179*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A179="","",IF(D179=0,"Check target/activation",IF(C179="Seed","P2 keep (seeding)",IF(H179&gt;=G179,"P2 hero - scale",IF(AND(B179="0→1 validate",F179&lt;50),"Learning - hold until ~50 conversions",IF(H179&gt;=G179*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
         <v/>
       </c>
       <c r="J180" s="6">
-        <f>IF(A180="","",IF(D180=0,"Check target/activation",IF(C180="Seed","P2 keep (seeding)",IF(H180&gt;=G180,"P2 hero - scale",IF(H180&gt;=G180*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A180="","",IF(D180=0,"Check target/activation",IF(C180="Seed","P2 keep (seeding)",IF(H180&gt;=G180,"P2 hero - scale",IF(AND(B180="0→1 validate",F180&lt;50),"Learning - hold until ~50 conversions",IF(H180&gt;=G180*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
         <v/>
       </c>
       <c r="J181" s="6">
-        <f>IF(A181="","",IF(D181=0,"Check target/activation",IF(C181="Seed","P2 keep (seeding)",IF(H181&gt;=G181,"P2 hero - scale",IF(H181&gt;=G181*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A181="","",IF(D181=0,"Check target/activation",IF(C181="Seed","P2 keep (seeding)",IF(H181&gt;=G181,"P2 hero - scale",IF(AND(B181="0→1 validate",F181&lt;50),"Learning - hold until ~50 conversions",IF(H181&gt;=G181*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
         <v/>
       </c>
       <c r="J182" s="6">
-        <f>IF(A182="","",IF(D182=0,"Check target/activation",IF(C182="Seed","P2 keep (seeding)",IF(H182&gt;=G182,"P2 hero - scale",IF(H182&gt;=G182*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A182="","",IF(D182=0,"Check target/activation",IF(C182="Seed","P2 keep (seeding)",IF(H182&gt;=G182,"P2 hero - scale",IF(AND(B182="0→1 validate",F182&lt;50),"Learning - hold until ~50 conversions",IF(H182&gt;=G182*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
         <v/>
       </c>
       <c r="J183" s="6">
-        <f>IF(A183="","",IF(D183=0,"Check target/activation",IF(C183="Seed","P2 keep (seeding)",IF(H183&gt;=G183,"P2 hero - scale",IF(H183&gt;=G183*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A183="","",IF(D183=0,"Check target/activation",IF(C183="Seed","P2 keep (seeding)",IF(H183&gt;=G183,"P2 hero - scale",IF(AND(B183="0→1 validate",F183&lt;50),"Learning - hold until ~50 conversions",IF(H183&gt;=G183*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
         <v/>
       </c>
       <c r="J184" s="6">
-        <f>IF(A184="","",IF(D184=0,"Check target/activation",IF(C184="Seed","P2 keep (seeding)",IF(H184&gt;=G184,"P2 hero - scale",IF(H184&gt;=G184*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A184="","",IF(D184=0,"Check target/activation",IF(C184="Seed","P2 keep (seeding)",IF(H184&gt;=G184,"P2 hero - scale",IF(AND(B184="0→1 validate",F184&lt;50),"Learning - hold until ~50 conversions",IF(H184&gt;=G184*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3677,7 +3677,7 @@
         <v/>
       </c>
       <c r="J185" s="6">
-        <f>IF(A185="","",IF(D185=0,"Check target/activation",IF(C185="Seed","P2 keep (seeding)",IF(H185&gt;=G185,"P2 hero - scale",IF(H185&gt;=G185*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A185="","",IF(D185=0,"Check target/activation",IF(C185="Seed","P2 keep (seeding)",IF(H185&gt;=G185,"P2 hero - scale",IF(AND(B185="0→1 validate",F185&lt;50),"Learning - hold until ~50 conversions",IF(H185&gt;=G185*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3694,7 +3694,7 @@
         <v/>
       </c>
       <c r="J186" s="6">
-        <f>IF(A186="","",IF(D186=0,"Check target/activation",IF(C186="Seed","P2 keep (seeding)",IF(H186&gt;=G186,"P2 hero - scale",IF(H186&gt;=G186*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A186="","",IF(D186=0,"Check target/activation",IF(C186="Seed","P2 keep (seeding)",IF(H186&gt;=G186,"P2 hero - scale",IF(AND(B186="0→1 validate",F186&lt;50),"Learning - hold until ~50 conversions",IF(H186&gt;=G186*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
         <v/>
       </c>
       <c r="J187" s="6">
-        <f>IF(A187="","",IF(D187=0,"Check target/activation",IF(C187="Seed","P2 keep (seeding)",IF(H187&gt;=G187,"P2 hero - scale",IF(H187&gt;=G187*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A187="","",IF(D187=0,"Check target/activation",IF(C187="Seed","P2 keep (seeding)",IF(H187&gt;=G187,"P2 hero - scale",IF(AND(B187="0→1 validate",F187&lt;50),"Learning - hold until ~50 conversions",IF(H187&gt;=G187*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3728,7 +3728,7 @@
         <v/>
       </c>
       <c r="J188" s="6">
-        <f>IF(A188="","",IF(D188=0,"Check target/activation",IF(C188="Seed","P2 keep (seeding)",IF(H188&gt;=G188,"P2 hero - scale",IF(H188&gt;=G188*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A188="","",IF(D188=0,"Check target/activation",IF(C188="Seed","P2 keep (seeding)",IF(H188&gt;=G188,"P2 hero - scale",IF(AND(B188="0→1 validate",F188&lt;50),"Learning - hold until ~50 conversions",IF(H188&gt;=G188*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
         <v/>
       </c>
       <c r="J189" s="6">
-        <f>IF(A189="","",IF(D189=0,"Check target/activation",IF(C189="Seed","P2 keep (seeding)",IF(H189&gt;=G189,"P2 hero - scale",IF(H189&gt;=G189*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A189="","",IF(D189=0,"Check target/activation",IF(C189="Seed","P2 keep (seeding)",IF(H189&gt;=G189,"P2 hero - scale",IF(AND(B189="0→1 validate",F189&lt;50),"Learning - hold until ~50 conversions",IF(H189&gt;=G189*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3762,7 +3762,7 @@
         <v/>
       </c>
       <c r="J190" s="6">
-        <f>IF(A190="","",IF(D190=0,"Check target/activation",IF(C190="Seed","P2 keep (seeding)",IF(H190&gt;=G190,"P2 hero - scale",IF(H190&gt;=G190*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A190="","",IF(D190=0,"Check target/activation",IF(C190="Seed","P2 keep (seeding)",IF(H190&gt;=G190,"P2 hero - scale",IF(AND(B190="0→1 validate",F190&lt;50),"Learning - hold until ~50 conversions",IF(H190&gt;=G190*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
         <v/>
       </c>
       <c r="J191" s="6">
-        <f>IF(A191="","",IF(D191=0,"Check target/activation",IF(C191="Seed","P2 keep (seeding)",IF(H191&gt;=G191,"P2 hero - scale",IF(H191&gt;=G191*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A191="","",IF(D191=0,"Check target/activation",IF(C191="Seed","P2 keep (seeding)",IF(H191&gt;=G191,"P2 hero - scale",IF(AND(B191="0→1 validate",F191&lt;50),"Learning - hold until ~50 conversions",IF(H191&gt;=G191*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3796,7 +3796,7 @@
         <v/>
       </c>
       <c r="J192" s="6">
-        <f>IF(A192="","",IF(D192=0,"Check target/activation",IF(C192="Seed","P2 keep (seeding)",IF(H192&gt;=G192,"P2 hero - scale",IF(H192&gt;=G192*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A192="","",IF(D192=0,"Check target/activation",IF(C192="Seed","P2 keep (seeding)",IF(H192&gt;=G192,"P2 hero - scale",IF(AND(B192="0→1 validate",F192&lt;50),"Learning - hold until ~50 conversions",IF(H192&gt;=G192*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
         <v/>
       </c>
       <c r="J193" s="6">
-        <f>IF(A193="","",IF(D193=0,"Check target/activation",IF(C193="Seed","P2 keep (seeding)",IF(H193&gt;=G193,"P2 hero - scale",IF(H193&gt;=G193*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A193="","",IF(D193=0,"Check target/activation",IF(C193="Seed","P2 keep (seeding)",IF(H193&gt;=G193,"P2 hero - scale",IF(AND(B193="0→1 validate",F193&lt;50),"Learning - hold until ~50 conversions",IF(H193&gt;=G193*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
         <v/>
       </c>
       <c r="J194" s="6">
-        <f>IF(A194="","",IF(D194=0,"Check target/activation",IF(C194="Seed","P2 keep (seeding)",IF(H194&gt;=G194,"P2 hero - scale",IF(H194&gt;=G194*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A194="","",IF(D194=0,"Check target/activation",IF(C194="Seed","P2 keep (seeding)",IF(H194&gt;=G194,"P2 hero - scale",IF(AND(B194="0→1 validate",F194&lt;50),"Learning - hold until ~50 conversions",IF(H194&gt;=G194*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
         <v/>
       </c>
       <c r="J195" s="6">
-        <f>IF(A195="","",IF(D195=0,"Check target/activation",IF(C195="Seed","P2 keep (seeding)",IF(H195&gt;=G195,"P2 hero - scale",IF(H195&gt;=G195*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A195="","",IF(D195=0,"Check target/activation",IF(C195="Seed","P2 keep (seeding)",IF(H195&gt;=G195,"P2 hero - scale",IF(AND(B195="0→1 validate",F195&lt;50),"Learning - hold until ~50 conversions",IF(H195&gt;=G195*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3864,7 +3864,7 @@
         <v/>
       </c>
       <c r="J196" s="6">
-        <f>IF(A196="","",IF(D196=0,"Check target/activation",IF(C196="Seed","P2 keep (seeding)",IF(H196&gt;=G196,"P2 hero - scale",IF(H196&gt;=G196*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A196="","",IF(D196=0,"Check target/activation",IF(C196="Seed","P2 keep (seeding)",IF(H196&gt;=G196,"P2 hero - scale",IF(AND(B196="0→1 validate",F196&lt;50),"Learning - hold until ~50 conversions",IF(H196&gt;=G196*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
         <v/>
       </c>
       <c r="J197" s="6">
-        <f>IF(A197="","",IF(D197=0,"Check target/activation",IF(C197="Seed","P2 keep (seeding)",IF(H197&gt;=G197,"P2 hero - scale",IF(H197&gt;=G197*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A197="","",IF(D197=0,"Check target/activation",IF(C197="Seed","P2 keep (seeding)",IF(H197&gt;=G197,"P2 hero - scale",IF(AND(B197="0→1 validate",F197&lt;50),"Learning - hold until ~50 conversions",IF(H197&gt;=G197*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3898,7 +3898,7 @@
         <v/>
       </c>
       <c r="J198" s="6">
-        <f>IF(A198="","",IF(D198=0,"Check target/activation",IF(C198="Seed","P2 keep (seeding)",IF(H198&gt;=G198,"P2 hero - scale",IF(H198&gt;=G198*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A198="","",IF(D198=0,"Check target/activation",IF(C198="Seed","P2 keep (seeding)",IF(H198&gt;=G198,"P2 hero - scale",IF(AND(B198="0→1 validate",F198&lt;50),"Learning - hold until ~50 conversions",IF(H198&gt;=G198*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
         <v/>
       </c>
       <c r="J199" s="6">
-        <f>IF(A199="","",IF(D199=0,"Check target/activation",IF(C199="Seed","P2 keep (seeding)",IF(H199&gt;=G199,"P2 hero - scale",IF(H199&gt;=G199*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A199="","",IF(D199=0,"Check target/activation",IF(C199="Seed","P2 keep (seeding)",IF(H199&gt;=G199,"P2 hero - scale",IF(AND(B199="0→1 validate",F199&lt;50),"Learning - hold until ~50 conversions",IF(H199&gt;=G199*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
         <v/>
       </c>
       <c r="J200" s="6">
-        <f>IF(A200="","",IF(D200=0,"Check target/activation",IF(C200="Seed","P2 keep (seeding)",IF(H200&gt;=G200,"P2 hero - scale",IF(H200&gt;=G200*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A200="","",IF(D200=0,"Check target/activation",IF(C200="Seed","P2 keep (seeding)",IF(H200&gt;=G200,"P2 hero - scale",IF(AND(B200="0→1 validate",F200&lt;50),"Learning - hold until ~50 conversions",IF(H200&gt;=G200*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -3949,7 +3949,7 @@
         <v/>
       </c>
       <c r="J201" s="6">
-        <f>IF(A201="","",IF(D201=0,"Check target/activation",IF(C201="Seed","P2 keep (seeding)",IF(H201&gt;=G201,"P2 hero - scale",IF(H201&gt;=G201*0.7,"P1 watch","P0 fix opening")))))</f>
+        <f>IF(A201="","",IF(D201=0,"Check target/activation",IF(C201="Seed","P2 keep (seeding)",IF(H201&gt;=G201,"P2 hero - scale",IF(AND(B201="0→1 validate",F201&lt;50),"Learning - hold until ~50 conversions",IF(H201&gt;=G201*0.7,"P1 watch","P0 fix opening"))))))</f>
         <v/>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Per creative: activation, ROAS vs break-even, triage. Diagnose in order: target → activation → creative → conversion path.</t>
+          <t>Per creative: activation, ROAS vs break-even, triage. Diagnose in order: target → activation → creative → conversion path. Stage-aware: in 0→1, below break-even is expected while the system learns (≈50 conversions); judge creatives, not ROI, until then.</t>
         </is>
       </c>
     </row>

</xml_diff>